<commit_message>
2035 LIO updated 11_03_25
</commit_message>
<xml_diff>
--- a/EnergyScope_LCA-ANNE_20_02_25/case_studies/SA_FINAL_03-03-2025/2035_steamlow5/output/LCA_Operation_final.xlsx
+++ b/EnergyScope_LCA-ANNE_20_02_25/case_studies/SA_FINAL_03-03-2025/2035_steamlow5/output/LCA_Operation_final.xlsx
@@ -577,52 +577,52 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.105942012751865</v>
+        <v>1.971562851151286e-08</v>
       </c>
       <c r="C3" t="n">
-        <v>1851.124675</v>
+        <v>3.299999999998503e-05</v>
       </c>
       <c r="D3" t="n">
-        <v>16905.31141967681</v>
+        <v>0.0003013709905028854</v>
       </c>
       <c r="E3" t="n">
-        <v>0.04497773120039218</v>
+        <v>8.018180242842199e-10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2574060794149415</v>
+        <v>4.588778235960372e-09</v>
       </c>
       <c r="G3" t="n">
-        <v>2.984053675000247</v>
+        <v>5.319672553927978e-08</v>
       </c>
       <c r="H3" t="n">
-        <v>1.32159111956965e-07</v>
+        <v>2.35600051875375e-15</v>
       </c>
       <c r="I3" t="n">
-        <v>3.422784378754294e-06</v>
+        <v>6.10179778943525e-14</v>
       </c>
       <c r="J3" t="n">
-        <v>17.91211470785053</v>
+        <v>3.193192729489166e-07</v>
       </c>
       <c r="K3" t="n">
-        <v>987.9160344710043</v>
+        <v>1.761157937000022e-05</v>
       </c>
       <c r="L3" t="n">
-        <v>0.002886676318740701</v>
+        <v>5.146077938721223e-11</v>
       </c>
       <c r="M3" t="n">
-        <v>1.045727863827076e-05</v>
+        <v>1.864219086500905e-13</v>
       </c>
       <c r="N3" t="n">
-        <v>1.120539610028009</v>
+        <v>1.997585988145695e-08</v>
       </c>
       <c r="O3" t="n">
-        <v>115.5761269200695</v>
+        <v>2.060375640749623e-06</v>
       </c>
       <c r="P3" t="n">
-        <v>5859.883498203973</v>
+        <v>0.0001044641444481007</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.709860257277062e-05</v>
+        <v>6.613567964571999e-13</v>
       </c>
     </row>
     <row r="4">
@@ -742,52 +742,52 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.794556105327804e-09</v>
+        <v>1.122695245407505e-09</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.0001599999999999654</v>
+        <v>-3.1e-05</v>
       </c>
       <c r="D6" t="n">
-        <v>0.00144464208132162</v>
+        <v>0.0002798994032561244</v>
       </c>
       <c r="E6" t="n">
-        <v>2.149806296832501e-10</v>
+        <v>4.165249700113871e-11</v>
       </c>
       <c r="F6" t="n">
-        <v>1.248608169862546e-09</v>
+        <v>2.419178329109205e-10</v>
       </c>
       <c r="G6" t="n">
-        <v>1.205128659686212e-08</v>
+        <v>2.334936778142541e-09</v>
       </c>
       <c r="H6" t="n">
-        <v>1.821185850354725e-15</v>
+        <v>3.528547585063042e-16</v>
       </c>
       <c r="I6" t="n">
-        <v>7.066984673740758e-14</v>
+        <v>1.369228280537568e-14</v>
       </c>
       <c r="J6" t="n">
-        <v>1.442593619323266e-07</v>
+        <v>2.795025137439432e-08</v>
       </c>
       <c r="K6" t="n">
-        <v>1.803588566974106e-05</v>
+        <v>3.494452848513085e-06</v>
       </c>
       <c r="L6" t="n">
-        <v>5.056426963761495e-11</v>
+        <v>9.796827242290013e-12</v>
       </c>
       <c r="M6" t="n">
-        <v>1.126676907702727e-13</v>
+        <v>2.182936508674505e-14</v>
       </c>
       <c r="N6" t="n">
-        <v>3.370961600920208e-09</v>
+        <v>6.531238101784313e-10</v>
       </c>
       <c r="O6" t="n">
-        <v>7.215455052691709e-07</v>
+        <v>1.397994416459321e-07</v>
       </c>
       <c r="P6" t="n">
-        <v>1.227674969094586e-05</v>
+        <v>2.378620252621273e-06</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.014124246198137e-13</v>
+        <v>1.964865727009315e-14</v>
       </c>
     </row>
     <row r="7">
@@ -907,52 +907,52 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.348466673854961e-07</v>
+        <v>2.838877208115938e-08</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0002279999999999815</v>
+        <v>4.8e-05</v>
       </c>
       <c r="D9" t="n">
-        <v>0.005595892655024286</v>
+        <v>0.001178082664215735</v>
       </c>
       <c r="E9" t="n">
-        <v>2.730580884563471e-09</v>
+        <v>5.748591335923563e-10</v>
       </c>
       <c r="F9" t="n">
-        <v>7.556952297486316e-08</v>
+        <v>1.590937325786722e-08</v>
       </c>
       <c r="G9" t="n">
-        <v>6.061770732181687e-07</v>
+        <v>1.276162259406775e-07</v>
       </c>
       <c r="H9" t="n">
-        <v>2.093278899292671e-14</v>
+        <v>4.406902945879664e-15</v>
       </c>
       <c r="I9" t="n">
-        <v>1.539645587324791e-12</v>
+        <v>3.241359131210349e-13</v>
       </c>
       <c r="J9" t="n">
-        <v>2.829602903361676e-07</v>
+        <v>5.9570587439198e-08</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0002765911290793911</v>
+        <v>5.822971138513969e-05</v>
       </c>
       <c r="L9" t="n">
-        <v>3.025749197902945e-10</v>
+        <v>6.369998311375138e-11</v>
       </c>
       <c r="M9" t="n">
-        <v>1.316051302044579e-12</v>
+        <v>2.770634320094075e-13</v>
       </c>
       <c r="N9" t="n">
-        <v>1.339028683550266e-07</v>
+        <v>2.819007754842895e-08</v>
       </c>
       <c r="O9" t="n">
-        <v>2.303753591127732e-05</v>
+        <v>4.850007560269302e-06</v>
       </c>
       <c r="P9" t="n">
-        <v>4.244085859896014e-05</v>
+        <v>8.934917599781807e-06</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.36176928325306e-13</v>
+        <v>1.760372480684997e-13</v>
       </c>
     </row>
     <row r="10">
@@ -962,52 +962,52 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7.799556816459215e-06</v>
+        <v>0.006979521687537082</v>
       </c>
       <c r="C10" t="n">
-        <v>0.07124899999999997</v>
+        <v>63.75797399999999</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3697759741372606</v>
+        <v>330.8982153415226</v>
       </c>
       <c r="E10" t="n">
-        <v>1.20124153518843e-07</v>
+        <v>0.0001074944582636445</v>
       </c>
       <c r="F10" t="n">
-        <v>4.487573838939184e-06</v>
+        <v>0.004015756237226695</v>
       </c>
       <c r="G10" t="n">
-        <v>3.003437015615707e-05</v>
+        <v>0.02687659604377098</v>
       </c>
       <c r="H10" t="n">
-        <v>1.916633294126634e-12</v>
+        <v>1.715120994462523e-09</v>
       </c>
       <c r="I10" t="n">
-        <v>4.663899968944512e-11</v>
+        <v>4.173543670206811e-08</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0001237160719830816</v>
+        <v>0.1107087271523733</v>
       </c>
       <c r="K10" t="n">
-        <v>0.02390789507362186</v>
+        <v>21.39425048069041</v>
       </c>
       <c r="L10" t="n">
-        <v>5.215430390344492e-09</v>
+        <v>4.667086909660402e-06</v>
       </c>
       <c r="M10" t="n">
-        <v>1.523290617301938e-10</v>
+        <v>1.363133848508484e-07</v>
       </c>
       <c r="N10" t="n">
-        <v>1.394564983933198e-05</v>
+        <v>0.01247942258655185</v>
       </c>
       <c r="O10" t="n">
-        <v>0.0007794543352592988</v>
+        <v>0.6975035332657255</v>
       </c>
       <c r="P10" t="n">
-        <v>0.02400108930103922</v>
+        <v>21.47764638980669</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.671749308729964e-10</v>
+        <v>3.28570642339574e-07</v>
       </c>
     </row>
     <row r="11">
@@ -1017,52 +1017,52 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5.529983980255294</v>
+        <v>5.4940350515228</v>
       </c>
       <c r="C11" t="n">
-        <v>10124.488538</v>
+        <v>10058.671979</v>
       </c>
       <c r="D11" t="n">
-        <v>244953.9226508398</v>
+        <v>243361.543515645</v>
       </c>
       <c r="E11" t="n">
-        <v>0.08758464913940346</v>
+        <v>0.0870152850469911</v>
       </c>
       <c r="F11" t="n">
-        <v>3.234807066731423</v>
+        <v>3.213778461744411</v>
       </c>
       <c r="G11" t="n">
-        <v>25.50710416112986</v>
+        <v>25.34128938247323</v>
       </c>
       <c r="H11" t="n">
-        <v>8.901230843854041e-07</v>
+        <v>8.843366351953213e-07</v>
       </c>
       <c r="I11" t="n">
-        <v>6.73013786979249e-05</v>
+        <v>6.686387065539733e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>12.22499127029902</v>
+        <v>12.14551991170187</v>
       </c>
       <c r="K11" t="n">
-        <v>12295.86944286457</v>
+        <v>12215.9373244563</v>
       </c>
       <c r="L11" t="n">
-        <v>0.009212451127385833</v>
+        <v>0.009152563476677903</v>
       </c>
       <c r="M11" t="n">
-        <v>5.818814730185179e-05</v>
+        <v>5.780988190942047e-05</v>
       </c>
       <c r="N11" t="n">
-        <v>5.2885112917223</v>
+        <v>5.254132111564469</v>
       </c>
       <c r="O11" t="n">
-        <v>690.1275130578979</v>
+        <v>685.6411809325548</v>
       </c>
       <c r="P11" t="n">
-        <v>1865.609302273875</v>
+        <v>1853.481481273021</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.672430060355626e-05</v>
+        <v>3.64855658676399e-05</v>
       </c>
     </row>
     <row r="12">
@@ -1072,52 +1072,52 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9.318904011093018e-08</v>
+        <v>3.727561604437207e-07</v>
       </c>
       <c r="C12" t="n">
-        <v>7.999999999999661e-06</v>
+        <v>3.199999999999864e-05</v>
       </c>
       <c r="D12" t="n">
-        <v>3.828515014643093e-07</v>
+        <v>1.531406005857237e-06</v>
       </c>
       <c r="E12" t="n">
-        <v>2.298794171088325e-13</v>
+        <v>9.1951766843533e-13</v>
       </c>
       <c r="F12" t="n">
-        <v>4.775821054319285e-08</v>
+        <v>1.910328421727714e-07</v>
       </c>
       <c r="G12" t="n">
-        <v>5.245887037777792e-07</v>
+        <v>2.098354815111117e-06</v>
       </c>
       <c r="H12" t="n">
-        <v>2.204959024346969e-17</v>
+        <v>8.819836097387875e-17</v>
       </c>
       <c r="I12" t="n">
-        <v>7.712040894528662e-15</v>
+        <v>3.084816357811465e-14</v>
       </c>
       <c r="J12" t="n">
-        <v>1.502428814834675e-09</v>
+        <v>6.009715259338699e-09</v>
       </c>
       <c r="K12" t="n">
-        <v>5.28052594639722e-08</v>
+        <v>2.112210378558888e-07</v>
       </c>
       <c r="L12" t="n">
-        <v>3.84768775562687e-14</v>
+        <v>1.539075102250748e-13</v>
       </c>
       <c r="M12" t="n">
-        <v>3.738732130281558e-14</v>
+        <v>1.495492852112623e-13</v>
       </c>
       <c r="N12" t="n">
-        <v>1.256633660625375e-07</v>
+        <v>5.026534642501501e-07</v>
       </c>
       <c r="O12" t="n">
-        <v>1.896392873711598e-09</v>
+        <v>7.58557149484639e-09</v>
       </c>
       <c r="P12" t="n">
-        <v>3.187475524827868e-07</v>
+        <v>1.274990209931147e-06</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.454255962524341e-15</v>
+        <v>2.181702385009736e-14</v>
       </c>
     </row>
     <row r="13">
@@ -1127,52 +1127,52 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9.99070985170658</v>
+        <v>9.990709152537269</v>
       </c>
       <c r="C13" t="n">
-        <v>857.3639889999999</v>
+        <v>857.363929</v>
       </c>
       <c r="D13" t="n">
-        <v>38.38107321215723</v>
+        <v>38.38107052617507</v>
       </c>
       <c r="E13" t="n">
-        <v>2.144124637767764e-05</v>
+        <v>2.144124487717751e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>5.120446226232636</v>
+        <v>5.120445867893848</v>
       </c>
       <c r="G13" t="n">
-        <v>56.24437902924326</v>
+        <v>56.24437509315219</v>
       </c>
       <c r="H13" t="n">
-        <v>2.30491346320365e-09</v>
+        <v>2.304913301901321e-09</v>
       </c>
       <c r="I13" t="n">
-        <v>8.256669727508741e-07</v>
+        <v>8.256669149690932e-07</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1401341050405628</v>
+        <v>0.1401340952337055</v>
       </c>
       <c r="K13" t="n">
-        <v>4.925236858714479</v>
+        <v>4.925236514036822</v>
       </c>
       <c r="L13" t="n">
-        <v>3.588804173525086e-06</v>
+        <v>3.588803922373588e-06</v>
       </c>
       <c r="M13" t="n">
-        <v>4.001280777710197e-06</v>
+        <v>4.001280497692785e-06</v>
       </c>
       <c r="N13" t="n">
-        <v>13.47300812628857</v>
+        <v>13.47300718342125</v>
       </c>
       <c r="O13" t="n">
-        <v>0.1768798065764722</v>
+        <v>0.1768797941980793</v>
       </c>
       <c r="P13" t="n">
-        <v>29.73012934789878</v>
+        <v>29.73012726732649</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.087277815918402e-07</v>
+        <v>5.087277459900804e-07</v>
       </c>
     </row>
     <row r="14">
@@ -1182,52 +1182,52 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.013983574937421e-08</v>
+        <v>2.807954515211397e-08</v>
       </c>
       <c r="C14" t="n">
-        <v>1.299999999999934e-05</v>
+        <v>3.599999999999915e-05</v>
       </c>
       <c r="D14" t="n">
-        <v>3.678122709863247e-07</v>
+        <v>1.018557058116004e-06</v>
       </c>
       <c r="E14" t="n">
-        <v>3.323312293529665e-13</v>
+        <v>9.203018659005479e-13</v>
       </c>
       <c r="F14" t="n">
-        <v>2.688700250346301e-09</v>
+        <v>7.445631462497653e-09</v>
       </c>
       <c r="G14" t="n">
-        <v>5.115336641882989e-08</v>
+        <v>1.416554762367636e-07</v>
       </c>
       <c r="H14" t="n">
-        <v>2.380316966361486e-17</v>
+        <v>6.591646983770449e-17</v>
       </c>
       <c r="I14" t="n">
-        <v>4.285377231802052e-15</v>
+        <v>1.186719848806755e-14</v>
       </c>
       <c r="J14" t="n">
-        <v>2.172025757267686e-09</v>
+        <v>6.014840558587601e-09</v>
       </c>
       <c r="K14" t="n">
-        <v>7.633931308688733e-08</v>
+        <v>2.114011747021553e-07</v>
       </c>
       <c r="L14" t="n">
-        <v>5.562511068272299e-14</v>
+        <v>1.540387680444679e-13</v>
       </c>
       <c r="M14" t="n">
-        <v>5.94294545306193e-14</v>
+        <v>1.645738740847964e-13</v>
       </c>
       <c r="N14" t="n">
-        <v>7.343874567396845e-09</v>
+        <v>2.03368834174072e-08</v>
       </c>
       <c r="O14" t="n">
-        <v>2.741570268144392e-09</v>
+        <v>7.592040742553907e-09</v>
       </c>
       <c r="P14" t="n">
-        <v>4.60805788089928e-07</v>
+        <v>1.276077567018297e-06</v>
       </c>
       <c r="Q14" t="n">
-        <v>7.885088678128826e-15</v>
+        <v>2.183563018558811e-14</v>
       </c>
     </row>
     <row r="15">
@@ -1237,52 +1237,52 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.425536386251619</v>
+        <v>4.425536838050888</v>
       </c>
       <c r="C15" t="n">
-        <v>3898.553178000001</v>
+        <v>3898.553576</v>
       </c>
       <c r="D15" t="n">
-        <v>1538.107980787521</v>
+        <v>1538.108137811665</v>
       </c>
       <c r="E15" t="n">
-        <v>0.00013339260157076</v>
+        <v>0.000133392615188698</v>
       </c>
       <c r="F15" t="n">
-        <v>2.215859332709232</v>
+        <v>2.215859558924438</v>
       </c>
       <c r="G15" t="n">
-        <v>25.08104288608404</v>
+        <v>25.08104544658651</v>
       </c>
       <c r="H15" t="n">
-        <v>3.437412785214505e-07</v>
+        <v>3.437413136137071e-07</v>
       </c>
       <c r="I15" t="n">
-        <v>1.70062077570225e-05</v>
+        <v>1.700620949317187e-05</v>
       </c>
       <c r="J15" t="n">
-        <v>0.06636743921068262</v>
+        <v>0.0663674459860784</v>
       </c>
       <c r="K15" t="n">
-        <v>5.086346159607235</v>
+        <v>5.086346678868017</v>
       </c>
       <c r="L15" t="n">
-        <v>4.738421867946343e-05</v>
+        <v>4.738422351687827e-05</v>
       </c>
       <c r="M15" t="n">
-        <v>7.227252829518035e-05</v>
+        <v>7.227253567342169e-05</v>
       </c>
       <c r="N15" t="n">
-        <v>6.011588409057334</v>
+        <v>6.011589022775315</v>
       </c>
       <c r="O15" t="n">
-        <v>0.924872740042474</v>
+        <v>0.9248728344619505</v>
       </c>
       <c r="P15" t="n">
-        <v>11.80862480349298</v>
+        <v>11.80862600902551</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.0001440494009082503</v>
+        <v>0.0001440494156141319</v>
       </c>
     </row>
     <row r="16">
@@ -1292,52 +1292,52 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.400130630901527e-08</v>
+        <v>3.266971472104247e-09</v>
       </c>
       <c r="C16" t="n">
-        <v>2.999999999999371e-05</v>
+        <v>6.999999999999999e-06</v>
       </c>
       <c r="D16" t="n">
-        <v>1.148995391837636e-05</v>
+        <v>2.680989247621712e-06</v>
       </c>
       <c r="E16" t="n">
-        <v>1.015480372730978e-12</v>
+        <v>2.369454203039446e-13</v>
       </c>
       <c r="F16" t="n">
-        <v>6.525037279476898e-09</v>
+        <v>1.522508698544928e-09</v>
       </c>
       <c r="G16" t="n">
-        <v>7.658110025854697e-08</v>
+        <v>1.78689233936647e-08</v>
       </c>
       <c r="H16" t="n">
-        <v>2.277609953200464e-15</v>
+        <v>5.31442322413553e-16</v>
       </c>
       <c r="I16" t="n">
-        <v>1.136670083606409e-13</v>
+        <v>2.652230195082177e-14</v>
       </c>
       <c r="J16" t="n">
-        <v>5.052366556560034e-10</v>
+        <v>1.178885529864255e-10</v>
       </c>
       <c r="K16" t="n">
-        <v>3.872092329840979e-08</v>
+        <v>9.034882102964179e-09</v>
       </c>
       <c r="L16" t="n">
-        <v>3.607227348412045e-13</v>
+        <v>8.416863812963202e-14</v>
       </c>
       <c r="M16" t="n">
-        <v>6.8919914412646e-13</v>
+        <v>1.60813133629541e-13</v>
       </c>
       <c r="N16" t="n">
-        <v>1.777378007009644e-08</v>
+        <v>4.147215349690038e-09</v>
       </c>
       <c r="O16" t="n">
-        <v>7.040796144071348e-09</v>
+        <v>1.642852433616992e-09</v>
       </c>
       <c r="P16" t="n">
-        <v>8.989574066092644e-08</v>
+        <v>2.097567282088723e-08</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.096607589952342e-12</v>
+        <v>2.558751043222668e-13</v>
       </c>
     </row>
     <row r="17">
@@ -1347,52 +1347,52 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3.221477877841433e-10</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>2.999999999999865e-06</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>1.646641291459944e-05</v>
+        <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>2.42561671613533e-12</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>1.973325284358553e-11</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>2.182311582633201e-10</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3.291821656634827e-16</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>9.962003246941898e-14</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>1.20682832526609e-09</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>9.249033397290351e-08</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>8.616366391875864e-13</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>5.90481535290548e-13</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1.115430984651279e-10</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>1.681792507326483e-08</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>2.147285335216186e-07</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.619400406603382e-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1402,52 +1402,52 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1.063578906951951e-10</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>9.999999999999551e-07</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>5.396255788355391e-06</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>8.085389053784432e-13</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>6.562179655867859e-12</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>7.253285304973089e-11</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>1.083217354445211e-16</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>3.264503302383228e-14</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>4.0227610842203e-10</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>3.083011132430117e-08</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>2.872122130625288e-13</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>1.933948757679974e-13</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>3.711759495911906e-11</v>
+        <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>5.605975024421609e-09</v>
+        <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>7.157617784053954e-08</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>8.73133468867794e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1457,52 +1457,52 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1.247753366467055e-08</v>
+        <v>1.848523505877383e-09</v>
       </c>
       <c r="C19" t="n">
-        <v>2.699999999999613e-05</v>
+        <v>4e-06</v>
       </c>
       <c r="D19" t="n">
-        <v>1.3826813919804e-05</v>
+        <v>2.048416877008293e-06</v>
       </c>
       <c r="E19" t="n">
-        <v>1.22559495452295e-12</v>
+        <v>1.815696228923148e-13</v>
       </c>
       <c r="F19" t="n">
-        <v>5.787697594313079e-09</v>
+        <v>8.574366806390975e-10</v>
       </c>
       <c r="G19" t="n">
-        <v>6.792840189829711e-08</v>
+        <v>1.006346694789731e-08</v>
       </c>
       <c r="H19" t="n">
-        <v>2.088787275509743e-15</v>
+        <v>3.094499667422285e-16</v>
       </c>
       <c r="I19" t="n">
-        <v>1.245495559826024e-13</v>
+        <v>1.84517860714993e-14</v>
       </c>
       <c r="J19" t="n">
-        <v>6.097759372214765e-10</v>
+        <v>9.033717588467611e-11</v>
       </c>
       <c r="K19" t="n">
-        <v>4.673272817806915e-08</v>
+        <v>6.923367137492718e-09</v>
       </c>
       <c r="L19" t="n">
-        <v>4.353604221952022e-13</v>
+        <v>6.449784032522438e-14</v>
       </c>
       <c r="M19" t="n">
-        <v>7.462099222385646e-13</v>
+        <v>1.105496181094328e-13</v>
       </c>
       <c r="N19" t="n">
-        <v>1.57743049994872e-08</v>
+        <v>2.336934073998438e-09</v>
       </c>
       <c r="O19" t="n">
-        <v>8.497617937008148e-09</v>
+        <v>1.258906361038424e-09</v>
       </c>
       <c r="P19" t="n">
-        <v>1.084962045015545e-07</v>
+        <v>1.607351177801037e-08</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.323508327120779e-12</v>
+        <v>1.960753077216249e-13</v>
       </c>
     </row>
     <row r="20">
@@ -1512,52 +1512,52 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1.489081879049019</v>
+        <v>1.489082205227204</v>
       </c>
       <c r="C20" t="n">
-        <v>465.654537</v>
+        <v>465.654639</v>
       </c>
       <c r="D20" t="n">
-        <v>11018.67133671018</v>
+        <v>11018.67375031165</v>
       </c>
       <c r="E20" t="n">
-        <v>0.04371132471220143</v>
+        <v>0.04371133428701444</v>
       </c>
       <c r="F20" t="n">
-        <v>0.3331144443687357</v>
+        <v>0.3331145173362912</v>
       </c>
       <c r="G20" t="n">
-        <v>2.603844018326998</v>
+        <v>2.603844588689936</v>
       </c>
       <c r="H20" t="n">
-        <v>4.195134831802043e-07</v>
+        <v>4.195135750731675e-07</v>
       </c>
       <c r="I20" t="n">
-        <v>2.658573901253592e-05</v>
+        <v>2.65857448360492e-05</v>
       </c>
       <c r="J20" t="n">
-        <v>33.87251709240759</v>
+        <v>33.87252451206415</v>
       </c>
       <c r="K20" t="n">
-        <v>4000.691400304181</v>
+        <v>4000.692276641659</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0209146644428748</v>
+        <v>0.020914669024159</v>
       </c>
       <c r="M20" t="n">
-        <v>7.665930653887517e-05</v>
+        <v>7.665932333082853e-05</v>
       </c>
       <c r="N20" t="n">
-        <v>1.171756879465269</v>
+        <v>1.171757136134521</v>
       </c>
       <c r="O20" t="n">
-        <v>230.3540187607163</v>
+        <v>230.3540692189595</v>
       </c>
       <c r="P20" t="n">
-        <v>5904.675032937399</v>
+        <v>5904.676326335842</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.0002629699400505569</v>
+        <v>0.0002629699976532038</v>
       </c>
     </row>
     <row r="21">
@@ -1567,52 +1567,52 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3.977734910676993e-09</v>
+        <v>4.972168638346242e-10</v>
       </c>
       <c r="C21" t="n">
-        <v>8e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="D21" t="n">
-        <v>1.13361426518003e-05</v>
+        <v>1.417017831475038e-06</v>
       </c>
       <c r="E21" t="n">
-        <v>4.327766060527198e-11</v>
+        <v>5.409707575658998e-12</v>
       </c>
       <c r="F21" t="n">
-        <v>1.017099981394455e-09</v>
+        <v>1.271374976743068e-10</v>
       </c>
       <c r="G21" t="n">
-        <v>1.505054234357945e-08</v>
+        <v>1.881317792947431e-09</v>
       </c>
       <c r="H21" t="n">
-        <v>4.709175912668435e-16</v>
+        <v>5.886469890835543e-17</v>
       </c>
       <c r="I21" t="n">
-        <v>3.071069648270466e-14</v>
+        <v>3.838837060338083e-15</v>
       </c>
       <c r="J21" t="n">
-        <v>3.352947408465985e-08</v>
+        <v>4.191184260582482e-09</v>
       </c>
       <c r="K21" t="n">
-        <v>3.959654497159019e-06</v>
+        <v>4.949568121448773e-07</v>
       </c>
       <c r="L21" t="n">
-        <v>2.070406195453359e-11</v>
+        <v>2.588007744316699e-12</v>
       </c>
       <c r="M21" t="n">
-        <v>1.069423310229e-13</v>
+        <v>1.33677913778625e-14</v>
       </c>
       <c r="N21" t="n">
-        <v>2.928253598764071e-09</v>
+        <v>3.660316998455089e-10</v>
       </c>
       <c r="O21" t="n">
-        <v>2.281105811257057e-07</v>
+        <v>2.851382264071321e-08</v>
       </c>
       <c r="P21" t="n">
-        <v>5.844920829176444e-06</v>
+        <v>7.306151036470555e-07</v>
       </c>
       <c r="Q21" t="n">
-        <v>2.874251970877444e-13</v>
+        <v>3.592814963596805e-14</v>
       </c>
     </row>
     <row r="22">
@@ -1622,52 +1622,52 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6.145243945712282e-09</v>
+        <v>1.659215865342735e-07</v>
       </c>
       <c r="C22" t="n">
-        <v>1.999999999999471e-06</v>
+        <v>5.399999999999933e-05</v>
       </c>
       <c r="D22" t="n">
-        <v>4.566613946925323e-05</v>
+        <v>0.001232985765670148</v>
       </c>
       <c r="E22" t="n">
-        <v>1.802844297947806e-10</v>
+        <v>4.867679604460305e-09</v>
       </c>
       <c r="F22" t="n">
-        <v>1.37393573799372e-09</v>
+        <v>3.70962649258398e-08</v>
       </c>
       <c r="G22" t="n">
-        <v>1.074104889131836e-08</v>
+        <v>2.90008320065669e-07</v>
       </c>
       <c r="H22" t="n">
-        <v>1.734982228165096e-15</v>
+        <v>4.684452016046942e-14</v>
       </c>
       <c r="I22" t="n">
-        <v>1.107681136249314e-13</v>
+        <v>2.990739067873901e-12</v>
       </c>
       <c r="J22" t="n">
-        <v>1.396837374305735e-07</v>
+        <v>3.771460910626436e-06</v>
       </c>
       <c r="K22" t="n">
-        <v>1.649650467296436e-05</v>
+        <v>0.0004454056261701503</v>
       </c>
       <c r="L22" t="n">
-        <v>8.625171682283348e-11</v>
+        <v>2.328796354217092e-09</v>
       </c>
       <c r="M22" t="n">
-        <v>3.233242285803662e-13</v>
+        <v>8.729754171672089e-12</v>
       </c>
       <c r="N22" t="n">
-        <v>4.834055295309561e-09</v>
+        <v>1.305194929733911e-07</v>
       </c>
       <c r="O22" t="n">
-        <v>9.502067986885981e-07</v>
+        <v>2.565558356459863e-05</v>
       </c>
       <c r="P22" t="n">
-        <v>2.434987984422511e-05</v>
+        <v>0.0006574467557942439</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.166637486320915e-12</v>
+        <v>3.149921213067265e-11</v>
       </c>
     </row>
     <row r="23">
@@ -1677,52 +1677,52 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1.874966474626158</v>
+        <v>1.874966542337661</v>
       </c>
       <c r="C23" t="n">
-        <v>3184.409391</v>
+        <v>3184.409506</v>
       </c>
       <c r="D23" t="n">
-        <v>3981.455769817273</v>
+        <v>3981.455913601365</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01515041642418863</v>
+        <v>0.01515041697132239</v>
       </c>
       <c r="F23" t="n">
-        <v>0.3214898692056808</v>
+        <v>0.3214898808157882</v>
       </c>
       <c r="G23" t="n">
-        <v>7.276364946799191</v>
+        <v>7.276365209573811</v>
       </c>
       <c r="H23" t="n">
-        <v>1.925243662034268e-07</v>
+        <v>1.925243731561453e-07</v>
       </c>
       <c r="I23" t="n">
-        <v>1.439090066623564e-05</v>
+        <v>1.439090118594067e-05</v>
       </c>
       <c r="J23" t="n">
-        <v>11.73753492034641</v>
+        <v>11.73753534422926</v>
       </c>
       <c r="K23" t="n">
-        <v>1386.119734692483</v>
+        <v>1386.119784750045</v>
       </c>
       <c r="L23" t="n">
-        <v>0.007247841667093475</v>
+        <v>0.007247841928838021</v>
       </c>
       <c r="M23" t="n">
-        <v>4.37197569885902e-05</v>
+        <v>4.371975856746133e-05</v>
       </c>
       <c r="N23" t="n">
-        <v>1.379676999712469</v>
+        <v>1.379677049537361</v>
       </c>
       <c r="O23" t="n">
-        <v>79.85748000851081</v>
+        <v>79.85748289243968</v>
       </c>
       <c r="P23" t="n">
-        <v>2046.110969534818</v>
+        <v>2046.111043426938</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.0001017333541920139</v>
+        <v>0.000101733357865956</v>
       </c>
     </row>
     <row r="24">
@@ -1732,52 +1732,52 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.248794418360026e-09</v>
+        <v>6.49758883672005e-10</v>
       </c>
       <c r="C24" t="n">
-        <v>5e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="D24" t="n">
-        <v>8.991656854150986e-06</v>
+        <v>1.798331370830197e-06</v>
       </c>
       <c r="E24" t="n">
-        <v>3.426015506055489e-11</v>
+        <v>6.852031012110978e-12</v>
       </c>
       <c r="F24" t="n">
-        <v>5.764808209275627e-10</v>
+        <v>1.152961641855125e-10</v>
       </c>
       <c r="G24" t="n">
-        <v>1.179812052638792e-08</v>
+        <v>2.359624105277583e-09</v>
       </c>
       <c r="H24" t="n">
-        <v>4.029166602337918e-16</v>
+        <v>8.058333204675834e-17</v>
       </c>
       <c r="I24" t="n">
-        <v>2.948920234161912e-14</v>
+        <v>5.897840468323822e-15</v>
       </c>
       <c r="J24" t="n">
-        <v>2.654248933763428e-08</v>
+        <v>5.308497867526854e-09</v>
       </c>
       <c r="K24" t="n">
-        <v>3.134479984803645e-06</v>
+        <v>6.26895996960729e-07</v>
       </c>
       <c r="L24" t="n">
-        <v>1.638979236059324e-11</v>
+        <v>3.277958472118647e-12</v>
       </c>
       <c r="M24" t="n">
-        <v>9.03823786258843e-14</v>
+        <v>1.807647572517686e-14</v>
       </c>
       <c r="N24" t="n">
-        <v>2.408867394805174e-09</v>
+        <v>4.817734789610348e-10</v>
       </c>
       <c r="O24" t="n">
-        <v>1.805844520199889e-07</v>
+        <v>3.611689040399777e-08</v>
       </c>
       <c r="P24" t="n">
-        <v>4.62694074701774e-06</v>
+        <v>9.253881494035477e-07</v>
       </c>
       <c r="Q24" t="n">
-        <v>2.300531148361096e-13</v>
+        <v>4.601062296722192e-14</v>
       </c>
     </row>
     <row r="25">
@@ -1787,52 +1787,52 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6.593103113404251e-09</v>
+        <v>1.198746020618955e-09</v>
       </c>
       <c r="C25" t="n">
-        <v>1.1e-05</v>
+        <v>2e-06</v>
       </c>
       <c r="D25" t="n">
-        <v>1.479920730720095e-05</v>
+        <v>2.690764964945627e-06</v>
       </c>
       <c r="E25" t="n">
-        <v>5.633167613819997e-11</v>
+        <v>1.024212293421818e-11</v>
       </c>
       <c r="F25" t="n">
-        <v>1.137898002586833e-09</v>
+        <v>2.068905459248787e-10</v>
       </c>
       <c r="G25" t="n">
-        <v>2.527739304556688e-08</v>
+        <v>4.595889644648523e-09</v>
       </c>
       <c r="H25" t="n">
-        <v>7.034518270828252e-16</v>
+        <v>1.279003321968773e-16</v>
       </c>
       <c r="I25" t="n">
-        <v>5.234215502374083e-14</v>
+        <v>9.516755458861969e-15</v>
       </c>
       <c r="J25" t="n">
-        <v>4.36420357884108e-08</v>
+        <v>7.934915597892871e-09</v>
       </c>
       <c r="K25" t="n">
-        <v>5.15381530099733e-06</v>
+        <v>9.370573274540599e-07</v>
       </c>
       <c r="L25" t="n">
-        <v>2.694863679389105e-11</v>
+        <v>4.899752144343827e-12</v>
       </c>
       <c r="M25" t="n">
-        <v>1.593191856607415e-13</v>
+        <v>2.896712466558936e-14</v>
       </c>
       <c r="N25" t="n">
-        <v>4.858449285027327e-09</v>
+        <v>8.833544154595139e-10</v>
       </c>
       <c r="O25" t="n">
-        <v>2.969229079320917e-07</v>
+        <v>5.39859832603803e-08</v>
       </c>
       <c r="P25" t="n">
-        <v>7.607768476557002e-06</v>
+        <v>1.383230632101273e-06</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.782609137823897e-13</v>
+        <v>6.877471159679811e-14</v>
       </c>
     </row>
     <row r="26">
@@ -1842,52 +1842,52 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>7.437402710181149e-09</v>
+        <v>8.263780789090165e-10</v>
       </c>
       <c r="C26" t="n">
-        <v>9e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="D26" t="n">
-        <v>1.620462407933762e-05</v>
+        <v>1.800513786593068e-06</v>
       </c>
       <c r="E26" t="n">
-        <v>6.166232051293226e-11</v>
+        <v>6.851368945881362e-12</v>
       </c>
       <c r="F26" t="n">
-        <v>1.285040133155433e-09</v>
+        <v>1.427822370172704e-10</v>
       </c>
       <c r="G26" t="n">
-        <v>2.914762715346209e-08</v>
+        <v>3.238625239273565e-09</v>
       </c>
       <c r="H26" t="n">
-        <v>6.062725371886182e-16</v>
+        <v>6.73636152431798e-17</v>
       </c>
       <c r="I26" t="n">
-        <v>4.912812190783913e-14</v>
+        <v>5.458680211982126e-15</v>
       </c>
       <c r="J26" t="n">
-        <v>4.777134089290806e-08</v>
+        <v>5.307926765878673e-09</v>
       </c>
       <c r="K26" t="n">
-        <v>5.641418027915796e-06</v>
+        <v>6.268242253239773e-07</v>
       </c>
       <c r="L26" t="n">
-        <v>2.949854305438998e-11</v>
+        <v>3.27761589493222e-12</v>
       </c>
       <c r="M26" t="n">
-        <v>1.752431724773054e-13</v>
+        <v>1.947146360858949e-14</v>
       </c>
       <c r="N26" t="n">
-        <v>4.615062897707627e-09</v>
+        <v>5.127847664119584e-10</v>
       </c>
       <c r="O26" t="n">
-        <v>3.250237462327186e-07</v>
+        <v>3.611374958141317e-08</v>
       </c>
       <c r="P26" t="n">
-        <v>8.327600733003988e-06</v>
+        <v>9.252889703337764e-07</v>
       </c>
       <c r="Q26" t="n">
-        <v>4.160826781608976e-13</v>
+        <v>4.623140868454418e-14</v>
       </c>
     </row>
     <row r="27">
@@ -1897,52 +1897,52 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5.086364272011055e-07</v>
+        <v>8.00541017859688e-08</v>
       </c>
       <c r="C27" t="n">
-        <v>0.0005209999999999978</v>
+        <v>8.199999999999787e-05</v>
       </c>
       <c r="D27" t="n">
-        <v>0.002411548779538318</v>
+        <v>0.0003795527829599574</v>
       </c>
       <c r="E27" t="n">
-        <v>9.428648877414662e-09</v>
+        <v>1.483971608345461e-09</v>
       </c>
       <c r="F27" t="n">
-        <v>1.002296980961699e-07</v>
+        <v>1.577511563125864e-08</v>
       </c>
       <c r="G27" t="n">
-        <v>1.439960221662298e-06</v>
+        <v>2.266348141579767e-07</v>
       </c>
       <c r="H27" t="n">
-        <v>9.717838497108902e-14</v>
+        <v>1.529487057126512e-14</v>
       </c>
       <c r="I27" t="n">
-        <v>6.531267245987595e-12</v>
+        <v>1.027953770001864e-12</v>
       </c>
       <c r="J27" t="n">
-        <v>7.304964564340371e-06</v>
+        <v>1.149725708782912e-06</v>
       </c>
       <c r="K27" t="n">
-        <v>0.0008626850006226016</v>
+        <v>0.0001357776776411743</v>
       </c>
       <c r="L27" t="n">
-        <v>4.510714462163924e-09</v>
+        <v>7.099397042177229e-10</v>
       </c>
       <c r="M27" t="n">
-        <v>1.930196973437143e-11</v>
+        <v>3.037929977386608e-12</v>
       </c>
       <c r="N27" t="n">
-        <v>3.865036666598618e-07</v>
+        <v>6.083167114416119e-08</v>
       </c>
       <c r="O27" t="n">
-        <v>4.969653445561751e-05</v>
+        <v>7.821719434473218e-06</v>
       </c>
       <c r="P27" t="n">
-        <v>0.001273414509187045</v>
+        <v>0.0002004222452079374</v>
       </c>
       <c r="Q27" t="n">
-        <v>6.224937381724218e-11</v>
+        <v>9.797406243788382e-12</v>
       </c>
     </row>
     <row r="28">
@@ -1952,52 +1952,52 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>9.673953618884987e-07</v>
+        <v>1.767829087714959e-07</v>
       </c>
       <c r="C28" t="n">
-        <v>0.002954999999999985</v>
+        <v>0.0005399999999999777</v>
       </c>
       <c r="D28" t="n">
-        <v>4.508313811333911e-05</v>
+        <v>8.238543005482993e-06</v>
       </c>
       <c r="E28" t="n">
-        <v>3.996413843569103e-09</v>
+        <v>7.30309128774023e-10</v>
       </c>
       <c r="F28" t="n">
-        <v>5.074640912910152e-07</v>
+        <v>9.273455475368471e-08</v>
       </c>
       <c r="G28" t="n">
-        <v>5.382525884962775e-06</v>
+        <v>9.836087911606748e-07</v>
       </c>
       <c r="H28" t="n">
-        <v>4.676388349718677e-14</v>
+        <v>8.545684293901843e-15</v>
       </c>
       <c r="I28" t="n">
-        <v>5.400642278740992e-13</v>
+        <v>9.869194011912116e-14</v>
       </c>
       <c r="J28" t="n">
-        <v>2.164763333179274e-07</v>
+        <v>3.955912690073657e-08</v>
       </c>
       <c r="K28" t="n">
-        <v>3.307336911459443e-05</v>
+        <v>6.043864406727698e-06</v>
       </c>
       <c r="L28" t="n">
-        <v>2.136516458060392e-11</v>
+        <v>3.904294035034078e-12</v>
       </c>
       <c r="M28" t="n">
-        <v>7.821569339315479e-12</v>
+        <v>1.429322315813945e-12</v>
       </c>
       <c r="N28" t="n">
-        <v>1.387431247940838e-06</v>
+        <v>2.535407356643064e-07</v>
       </c>
       <c r="O28" t="n">
-        <v>7.591923212776148e-06</v>
+        <v>1.387356526192546e-06</v>
       </c>
       <c r="P28" t="n">
-        <v>1.194828542064512e-05</v>
+        <v>2.183443021031516e-06</v>
       </c>
       <c r="Q28" t="n">
-        <v>2.225576565353056e-13</v>
+        <v>4.067043469680564e-14</v>
       </c>
     </row>
     <row r="29">
@@ -2007,52 +2007,52 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1.703377888516291e-08</v>
+        <v>0</v>
       </c>
       <c r="C29" t="n">
-        <v>9.999999999998096e-07</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>2.423979816128176e-06</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>1.894846653556111e-10</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>4.180407741162255e-09</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>8.321013252972704e-08</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>3.053535418483358e-16</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>1.041449016423711e-14</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>1.000244025029983e-08</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>1.550455442912187e-06</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>8.693495803304271e-13</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>8.287070894033722e-14</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
-        <v>7.948021550321779e-09</v>
+        <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.569058175767541e-07</v>
+        <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>5.4820251964944e-07</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>2.18515318691236e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2227,52 +2227,52 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1.635523202750225e-07</v>
+        <v>2.238317662300273e-08</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0007379999999999646</v>
+        <v>0.0001009999999999875</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0009589219326174845</v>
+        <v>0.0001312345734340902</v>
       </c>
       <c r="E33" t="n">
-        <v>1.588128735131119e-09</v>
+        <v>2.173455315016678e-10</v>
       </c>
       <c r="F33" t="n">
-        <v>2.40415166545941e-07</v>
+        <v>3.290234664110867e-08</v>
       </c>
       <c r="G33" t="n">
-        <v>7.385188012513676e-07</v>
+        <v>1.010710012552608e-07</v>
       </c>
       <c r="H33" t="n">
-        <v>2.545043233584935e-14</v>
+        <v>3.483053747859877e-15</v>
       </c>
       <c r="I33" t="n">
-        <v>3.045073654516024e-13</v>
+        <v>4.167377223659825e-14</v>
       </c>
       <c r="J33" t="n">
-        <v>3.709505460079891e-06</v>
+        <v>5.076694464336591e-07</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0002021951045456407</v>
+        <v>2.767168774946904e-05</v>
       </c>
       <c r="L33" t="n">
-        <v>2.712451723124184e-10</v>
+        <v>3.712162927310592e-11</v>
       </c>
       <c r="M33" t="n">
-        <v>8.606485630510071e-13</v>
+        <v>1.177852369487061e-13</v>
       </c>
       <c r="N33" t="n">
-        <v>1.831821873355442e-07</v>
+        <v>2.506964894429344e-08</v>
       </c>
       <c r="O33" t="n">
-        <v>6.119159750882956e-06</v>
+        <v>8.374459821668449e-07</v>
       </c>
       <c r="P33" t="n">
-        <v>5.779342548736108e-05</v>
+        <v>7.90939833905559e-06</v>
       </c>
       <c r="Q33" t="n">
-        <v>6.725248653869327e-13</v>
+        <v>9.203931084563013e-14</v>
       </c>
     </row>
     <row r="34">
@@ -2282,52 +2282,52 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>7.54784528133015e-08</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>1.999999999999935e-06</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0004695366337216702</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>7.77712545005864e-10</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>1.177322007318352e-07</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>3.616554022041929e-07</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1.246317131953335e-14</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>1.368335689734517e-13</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>1.816558612821582e-06</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>9.901569429819181e-05</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1.328297691573652e-10</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>3.93287371080215e-13</v>
+        <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>8.41818134339029e-08</v>
+        <v>0</v>
       </c>
       <c r="O34" t="n">
-        <v>2.996575276225151e-06</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>2.830165529161051e-05</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>3.293379264978887e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2337,28 +2337,28 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8.847695427532569e-08</v>
+        <v>1.832736909988584e-08</v>
       </c>
       <c r="C35" t="n">
-        <v>0.0002799999999999897</v>
+        <v>5.799999999998822e-05</v>
       </c>
       <c r="D35" t="n">
-        <v>2.454704324199497e-07</v>
+        <v>5.084744671555256e-08</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>4.462125076109482e-08</v>
+        <v>9.242973371939531e-09</v>
       </c>
       <c r="G35" t="n">
-        <v>4.886543422989289e-07</v>
+        <v>1.01221256619047e-07</v>
       </c>
       <c r="H35" t="n">
-        <v>1.384285579749408e-14</v>
+        <v>2.86744870090901e-15</v>
       </c>
       <c r="I35" t="n">
-        <v>9.662896203003726e-14</v>
+        <v>2.001599927764724e-14</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2370,10 +2370,10 @@
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>3.244214862515095e-13</v>
+        <v>6.720159358065866e-14</v>
       </c>
       <c r="N35" t="n">
-        <v>1.269820210820837e-07</v>
+        <v>2.630341865271296e-08</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
@@ -2392,28 +2392,28 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>5.632795939335677e-07</v>
+        <v>1.051987894107339e-07</v>
       </c>
       <c r="C36" t="n">
-        <v>0.0004229999999999952</v>
+        <v>7.899999999997887e-05</v>
       </c>
       <c r="D36" t="n">
-        <v>0.000148065175379272</v>
+        <v>2.765283417248107e-05</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1.10952170566154e-07</v>
+        <v>2.072156377003291e-08</v>
       </c>
       <c r="G36" t="n">
-        <v>1.225710937759392e-06</v>
+        <v>2.28915281520017e-07</v>
       </c>
       <c r="H36" t="n">
-        <v>1.332346821217245e-13</v>
+        <v>2.488307302036298e-14</v>
       </c>
       <c r="I36" t="n">
-        <v>6.119798986504391e-13</v>
+        <v>1.142941181876414e-13</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
@@ -2425,10 +2425,10 @@
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>2.740027582435751e-12</v>
+        <v>5.117309196509903e-13</v>
       </c>
       <c r="N36" t="n">
-        <v>3.143899977688163e-07</v>
+        <v>5.871586246744711e-08</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
@@ -2447,52 +2447,52 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>7.565618016868277e-07</v>
+        <v>1.460362132770227e-07</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0008029999999999586</v>
+        <v>0.0001549999999999801</v>
       </c>
       <c r="D37" t="n">
-        <v>0.01099973061164788</v>
+        <v>0.00212323567223573</v>
       </c>
       <c r="E37" t="n">
-        <v>1.150117432734879e-09</v>
+        <v>2.220027423087079e-10</v>
       </c>
       <c r="F37" t="n">
-        <v>3.641799173147369e-07</v>
+        <v>7.029624804953908e-08</v>
       </c>
       <c r="G37" t="n">
-        <v>4.155537095692672e-06</v>
+        <v>8.021273347849496e-07</v>
       </c>
       <c r="H37" t="n">
-        <v>8.92510044457447e-14</v>
+        <v>1.722777794407144e-14</v>
       </c>
       <c r="I37" t="n">
-        <v>5.126166454777815e-12</v>
+        <v>9.894841849196763e-13</v>
       </c>
       <c r="J37" t="n">
-        <v>3.47478819789599e-09</v>
+        <v>6.707249946124992e-10</v>
       </c>
       <c r="K37" t="n">
-        <v>1.726054089483209e-06</v>
+        <v>3.331735789164095e-07</v>
       </c>
       <c r="L37" t="n">
-        <v>8.85576761386232e-13</v>
+        <v>1.709394744892346e-13</v>
       </c>
       <c r="M37" t="n">
-        <v>1.874486886607411e-11</v>
+        <v>3.618249905655371e-12</v>
       </c>
       <c r="N37" t="n">
-        <v>9.868265854988158e-07</v>
+        <v>1.904833384213009e-07</v>
       </c>
       <c r="O37" t="n">
-        <v>2.674069567383326e-05</v>
+        <v>5.161653585857827e-06</v>
       </c>
       <c r="P37" t="n">
-        <v>6.316212082147925e-07</v>
+        <v>1.219194112992345e-07</v>
       </c>
       <c r="Q37" t="n">
-        <v>9.318892302930639e-15</v>
+        <v>1.798789921487096e-15</v>
       </c>
     </row>
     <row r="38">
@@ -2502,52 +2502,52 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>9.086009050302043e-07</v>
+        <v>1.412014919979261e-07</v>
       </c>
       <c r="C38" t="n">
-        <v>0.001035999999999963</v>
+        <v>0.0001609999999999816</v>
       </c>
       <c r="D38" t="n">
-        <v>4.492959577409668e-05</v>
+        <v>6.982302045973938e-06</v>
       </c>
       <c r="E38" t="n">
-        <v>1.915096457924512e-10</v>
+        <v>2.976163414341914e-11</v>
       </c>
       <c r="F38" t="n">
-        <v>4.715034702395979e-07</v>
+        <v>7.327418794263449e-08</v>
       </c>
       <c r="G38" t="n">
-        <v>5.137953985198527e-06</v>
+        <v>7.984658220240329e-07</v>
       </c>
       <c r="H38" t="n">
-        <v>8.647225264024668e-16</v>
+        <v>1.343825547787512e-16</v>
       </c>
       <c r="I38" t="n">
-        <v>3.018351955569586e-12</v>
+        <v>4.69068209311453e-13</v>
       </c>
       <c r="J38" t="n">
-        <v>1.321947927676374e-07</v>
+        <v>2.054378536253664e-08</v>
       </c>
       <c r="K38" t="n">
-        <v>6.284417974282342e-05</v>
+        <v>9.766325230302876e-06</v>
       </c>
       <c r="L38" t="n">
-        <v>1.609631383976651e-11</v>
+        <v>2.501454177801357e-12</v>
       </c>
       <c r="M38" t="n">
-        <v>2.683168936201503e-12</v>
+        <v>4.169789563015523e-13</v>
       </c>
       <c r="N38" t="n">
-        <v>1.524622720366237e-06</v>
+        <v>2.369346119487886e-07</v>
       </c>
       <c r="O38" t="n">
-        <v>2.538640318525546e-06</v>
+        <v>3.945184278789392e-07</v>
       </c>
       <c r="P38" t="n">
-        <v>2.51742993291396e-05</v>
+        <v>3.912222193041659e-06</v>
       </c>
       <c r="Q38" t="n">
-        <v>3.210770184462613e-13</v>
+        <v>4.989710421799616e-14</v>
       </c>
     </row>
     <row r="39">
@@ -2557,52 +2557,52 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1.159215955140636e-05</v>
+        <v>1.751746653928082e-06</v>
       </c>
       <c r="C39" t="n">
-        <v>0.001210999999999997</v>
+        <v>0.0001829999999999602</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0002351710257262731</v>
+        <v>3.553781809075036e-05</v>
       </c>
       <c r="E39" t="n">
-        <v>6.214543823029068e-10</v>
+        <v>9.391094299042727e-11</v>
       </c>
       <c r="F39" t="n">
-        <v>1.368515760619993e-06</v>
+        <v>2.068029596972789e-07</v>
       </c>
       <c r="G39" t="n">
-        <v>1.362731225143193e-05</v>
+        <v>2.059288308845174e-06</v>
       </c>
       <c r="H39" t="n">
-        <v>3.505887784348374e-13</v>
+        <v>5.29791465347328e-14</v>
       </c>
       <c r="I39" t="n">
-        <v>9.602729565181537e-13</v>
+        <v>1.451114376901604e-13</v>
       </c>
       <c r="J39" t="n">
-        <v>2.325376158811903e-07</v>
+        <v>3.513987093827303e-08</v>
       </c>
       <c r="K39" t="n">
-        <v>1.162623507175601e-05</v>
+        <v>1.756895968729059e-06</v>
       </c>
       <c r="L39" t="n">
-        <v>2.109682953626608e-11</v>
+        <v>3.188042778807481e-12</v>
       </c>
       <c r="M39" t="n">
-        <v>7.745781121921149e-11</v>
+        <v>1.170502019249599e-11</v>
       </c>
       <c r="N39" t="n">
-        <v>3.801791517673419e-06</v>
+        <v>5.745068932568832e-07</v>
       </c>
       <c r="O39" t="n">
-        <v>9.22479955317523e-06</v>
+        <v>1.394003565838731e-06</v>
       </c>
       <c r="P39" t="n">
-        <v>4.888457367076445e-05</v>
+        <v>7.387181652971069e-06</v>
       </c>
       <c r="Q39" t="n">
-        <v>4.282867768608523e-13</v>
+        <v>6.472046256442533e-14</v>
       </c>
     </row>
     <row r="40">
@@ -2667,52 +2667,52 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.03687068047500326</v>
+        <v>0.03624524340052928</v>
       </c>
       <c r="C41" t="n">
-        <v>1167.702872</v>
+        <v>1147.895137</v>
       </c>
       <c r="D41" t="n">
-        <v>197.9662645870648</v>
+        <v>194.6081643357874</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0006455744248470619</v>
+        <v>0.0006346235507533411</v>
       </c>
       <c r="F41" t="n">
-        <v>0.004658501992289444</v>
+        <v>0.004579479858172229</v>
       </c>
       <c r="G41" t="n">
-        <v>0.04862078461925516</v>
+        <v>0.04779603061691141</v>
       </c>
       <c r="H41" t="n">
-        <v>2.599695728158231e-08</v>
+        <v>2.555597109152702e-08</v>
       </c>
       <c r="I41" t="n">
-        <v>2.548665683766695e-07</v>
+        <v>2.505432687018833e-07</v>
       </c>
       <c r="J41" t="n">
-        <v>0.3211956352337958</v>
+        <v>0.3157471960987863</v>
       </c>
       <c r="K41" t="n">
-        <v>24.61617029651883</v>
+        <v>24.19860638566436</v>
       </c>
       <c r="L41" t="n">
-        <v>0.0002293233609706238</v>
+        <v>0.0002254333505301806</v>
       </c>
       <c r="M41" t="n">
-        <v>5.142211765664184e-07</v>
+        <v>5.054984466313875e-07</v>
       </c>
       <c r="N41" t="n">
-        <v>0.02666166607848399</v>
+        <v>0.0262094044381263</v>
       </c>
       <c r="O41" t="n">
-        <v>4.476066739675366</v>
+        <v>4.400139253370609</v>
       </c>
       <c r="P41" t="n">
-        <v>57.14969253152955</v>
+        <v>56.18026272867468</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.0006971496773123336</v>
+        <v>0.0006853239326005073</v>
       </c>
     </row>
     <row r="42">
@@ -2777,28 +2777,28 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.1849746611917859</v>
+        <v>0.2046943524891729</v>
       </c>
       <c r="C43" t="n">
-        <v>1302.899046</v>
+        <v>1441.797892</v>
       </c>
       <c r="D43" t="n">
-        <v>1.13647404967691</v>
+        <v>1.257630738288892</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>0.08995850620964149</v>
+        <v>0.09954876014279469</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9774612365620091</v>
+        <v>1.081665962311878</v>
       </c>
       <c r="H43" t="n">
-        <v>6.433070188205258e-08</v>
+        <v>7.118883895815198e-08</v>
       </c>
       <c r="I43" t="n">
-        <v>2.458683900127909e-07</v>
+        <v>2.720798111858283e-07</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2810,10 +2810,10 @@
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>1.012594011123556e-06</v>
+        <v>1.120544155106986e-06</v>
       </c>
       <c r="N43" t="n">
-        <v>0.2778353007661721</v>
+        <v>0.3074546352594789</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
@@ -2887,28 +2887,28 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>6.288183535996488e-08</v>
+        <v>9.79566279476424e-09</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0001989999999999967</v>
+        <v>3.099999999998633e-05</v>
       </c>
       <c r="D45" t="n">
-        <v>1.74459343041325e-07</v>
+        <v>2.71770835893406e-08</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>3.171296036235017e-08</v>
+        <v>4.940209905690643e-09</v>
       </c>
       <c r="G45" t="n">
-        <v>3.472936218481744e-07</v>
+        <v>5.410101646878812e-08</v>
       </c>
       <c r="H45" t="n">
-        <v>9.838315370362061e-15</v>
+        <v>1.532601891864796e-15</v>
       </c>
       <c r="I45" t="n">
-        <v>6.867558372849213e-14</v>
+        <v>1.069820651046408e-14</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2920,10 +2920,10 @@
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>2.305709848716132e-13</v>
+        <v>3.591809312068831e-14</v>
       </c>
       <c r="N45" t="n">
-        <v>9.02479364119113e-08</v>
+        <v>1.405872376265358e-08</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
@@ -2942,28 +2942,28 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2.876321330724307e-07</v>
+        <v>5.592847031963723e-08</v>
       </c>
       <c r="C46" t="n">
-        <v>0.0002159999999999755</v>
+        <v>4.199999999999367e-05</v>
       </c>
       <c r="D46" t="n">
-        <v>7.560774912983332e-05</v>
+        <v>1.470150677524482e-05</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>5.665642752313668e-08</v>
+        <v>1.101652757394283e-08</v>
       </c>
       <c r="G46" t="n">
-        <v>6.258949469409023e-07</v>
+        <v>1.217017952385042e-07</v>
       </c>
       <c r="H46" t="n">
-        <v>6.803473129619279e-14</v>
+        <v>1.322897552981477e-14</v>
       </c>
       <c r="I46" t="n">
-        <v>3.125003737789157e-13</v>
+        <v>6.076396156812024e-14</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
@@ -2975,10 +2975,10 @@
         <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>1.399163020818113e-12</v>
+        <v>2.720594762701785e-13</v>
       </c>
       <c r="N46" t="n">
-        <v>1.605395733287409e-07</v>
+        <v>3.121602814725402e-08</v>
       </c>
       <c r="O46" t="n">
         <v>0</v>
@@ -2997,52 +2997,52 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3.504869118648701e-07</v>
+        <v>7.820003678703264e-08</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0003719999999999685</v>
+        <v>8.299999999996997e-05</v>
       </c>
       <c r="D47" t="n">
-        <v>0.005095765613365979</v>
+        <v>0.00113695845674532</v>
       </c>
       <c r="E47" t="n">
-        <v>5.32806581540923e-10</v>
+        <v>1.188788878168934e-10</v>
       </c>
       <c r="F47" t="n">
-        <v>1.687109953189013e-07</v>
+        <v>3.7642507020067e-08</v>
       </c>
       <c r="G47" t="n">
-        <v>1.925105603483964e-06</v>
+        <v>4.295262502395825e-07</v>
       </c>
       <c r="H47" t="n">
-        <v>4.134666706577327e-14</v>
+        <v>9.225197221661908e-15</v>
       </c>
       <c r="I47" t="n">
-        <v>2.374762043807328e-12</v>
+        <v>5.298528216020258e-13</v>
       </c>
       <c r="J47" t="n">
-        <v>1.609739987070069e-09</v>
+        <v>3.591624164698352e-10</v>
       </c>
       <c r="K47" t="n">
-        <v>7.996165893994161e-07</v>
+        <v>1.784090777422933e-07</v>
       </c>
       <c r="L47" t="n">
-        <v>4.10254738774181e-13</v>
+        <v>9.153533150066553e-14</v>
       </c>
       <c r="M47" t="n">
-        <v>8.683799773573273e-12</v>
+        <v>1.937514465608553e-12</v>
       </c>
       <c r="N47" t="n">
-        <v>4.571600122111424e-07</v>
+        <v>1.020007554126728e-07</v>
       </c>
       <c r="O47" t="n">
-        <v>1.238796860605933e-05</v>
+        <v>2.76398224274903e-06</v>
       </c>
       <c r="P47" t="n">
-        <v>2.926065871181757e-07</v>
+        <v>6.528587830860711e-08</v>
       </c>
       <c r="Q47" t="n">
-        <v>4.317095811569222e-15</v>
+        <v>9.632229902154463e-16</v>
       </c>
     </row>
     <row r="48">
@@ -3052,52 +3052,52 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2.309392760773635e-07</v>
+        <v>4.381924725570916e-08</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0003899999999999617</v>
+        <v>7.4e-05</v>
       </c>
       <c r="D48" t="n">
-        <v>0.008127435952987282</v>
+        <v>0.001542128873131071</v>
       </c>
       <c r="E48" t="n">
-        <v>2.91518427920993e-09</v>
+        <v>5.531375299014256e-10</v>
       </c>
       <c r="F48" t="n">
-        <v>1.319528781561582e-07</v>
+        <v>2.503721277835042e-08</v>
       </c>
       <c r="G48" t="n">
-        <v>1.114729236555931e-06</v>
+        <v>2.115127269362744e-07</v>
       </c>
       <c r="H48" t="n">
-        <v>2.957047156909372e-14</v>
+        <v>5.610807425931155e-15</v>
       </c>
       <c r="I48" t="n">
-        <v>2.390205925655242e-12</v>
+        <v>4.535262525602699e-13</v>
       </c>
       <c r="J48" t="n">
-        <v>4.124136431002904e-07</v>
+        <v>7.825284510108842e-08</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0004111383369686828</v>
+        <v>7.801086393765517e-05</v>
       </c>
       <c r="L48" t="n">
-        <v>3.064173588513474e-10</v>
+        <v>5.814072962821008e-11</v>
       </c>
       <c r="M48" t="n">
-        <v>2.070394712726246e-12</v>
+        <v>3.928441249788647e-13</v>
       </c>
       <c r="N48" t="n">
-        <v>2.551412772731406e-07</v>
+        <v>4.841142184157501e-08</v>
       </c>
       <c r="O48" t="n">
-        <v>2.302417577199986e-05</v>
+        <v>4.368689761867068e-06</v>
       </c>
       <c r="P48" t="n">
-        <v>6.319835122484175e-05</v>
+        <v>1.199148202727884e-05</v>
       </c>
       <c r="Q48" t="n">
-        <v>1.23492883233562e-12</v>
+        <v>2.343198297252432e-13</v>
       </c>
     </row>
     <row r="49">
@@ -3107,52 +3107,52 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5.932617317994898</v>
+        <v>4.610306029004421</v>
       </c>
       <c r="C49" t="n">
-        <v>6764.456768</v>
+        <v>5256.738155999999</v>
       </c>
       <c r="D49" t="n">
-        <v>293.3632318702736</v>
+        <v>227.9759849800762</v>
       </c>
       <c r="E49" t="n">
-        <v>0.001250442779554127</v>
+        <v>0.0009717336508487059</v>
       </c>
       <c r="F49" t="n">
-        <v>3.078634015828041</v>
+        <v>2.392442357813701</v>
       </c>
       <c r="G49" t="n">
-        <v>33.54774865719113</v>
+        <v>26.07034629128025</v>
       </c>
       <c r="H49" t="n">
-        <v>5.64611790170409e-09</v>
+        <v>4.387663995070202e-09</v>
       </c>
       <c r="I49" t="n">
-        <v>1.97080225039184e-05</v>
+        <v>1.531533387362976e-05</v>
       </c>
       <c r="J49" t="n">
-        <v>0.863152471651964</v>
+        <v>0.6707658408939937</v>
       </c>
       <c r="K49" t="n">
-        <v>410.3346882150249</v>
+        <v>318.8758663481024</v>
       </c>
       <c r="L49" t="n">
-        <v>0.0001050992462290199</v>
+        <v>8.167384858345032e-05</v>
       </c>
       <c r="M49" t="n">
-        <v>1.751947902526667e-05</v>
+        <v>1.361459124124023e-05</v>
       </c>
       <c r="N49" t="n">
-        <v>9.954869188637391</v>
+        <v>7.736044814337844</v>
       </c>
       <c r="O49" t="n">
-        <v>16.57579409668768</v>
+        <v>12.88124268991671</v>
       </c>
       <c r="P49" t="n">
-        <v>164.3730303828788</v>
+        <v>127.7361967510214</v>
       </c>
       <c r="Q49" t="n">
-        <v>2.096439778453814e-06</v>
+        <v>1.629167774016639e-06</v>
       </c>
     </row>
     <row r="50">
@@ -3162,52 +3162,52 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6.290225121747518e-08</v>
+        <v>1.09395219508665e-08</v>
       </c>
       <c r="C50" t="n">
-        <v>0.0002989999999999658</v>
+        <v>5.199999999999999e-05</v>
       </c>
       <c r="D50" t="n">
-        <v>0.0006518567372615925</v>
+        <v>0.0001133663890889856</v>
       </c>
       <c r="E50" t="n">
-        <v>5.032929246680341e-10</v>
+        <v>8.752920429010289e-11</v>
       </c>
       <c r="F50" t="n">
-        <v>3.746067590655686e-08</v>
+        <v>6.514900157662806e-09</v>
       </c>
       <c r="G50" t="n">
-        <v>3.151481255287757e-07</v>
+        <v>5.480836965718463e-08</v>
       </c>
       <c r="H50" t="n">
-        <v>1.53283994589455e-14</v>
+        <v>2.665808601556043e-15</v>
       </c>
       <c r="I50" t="n">
-        <v>8.098756358520573e-13</v>
+        <v>1.408479366699391e-13</v>
       </c>
       <c r="J50" t="n">
-        <v>1.691306103075458e-07</v>
+        <v>2.941401918392437e-08</v>
       </c>
       <c r="K50" t="n">
-        <v>1.042899599006769e-05</v>
+        <v>1.813738433055457e-06</v>
       </c>
       <c r="L50" t="n">
-        <v>1.965606427171732e-11</v>
+        <v>3.418445960299056e-12</v>
       </c>
       <c r="M50" t="n">
-        <v>2.392934549926149e-13</v>
+        <v>4.161625304219865e-14</v>
       </c>
       <c r="N50" t="n">
-        <v>7.486363664789458e-08</v>
+        <v>1.30197628952875e-08</v>
       </c>
       <c r="O50" t="n">
-        <v>2.018504347954183e-05</v>
+        <v>3.510442344268546e-06</v>
       </c>
       <c r="P50" t="n">
-        <v>2.488085853918103e-05</v>
+        <v>4.327105832901543e-06</v>
       </c>
       <c r="Q50" t="n">
-        <v>4.67844636826024e-13</v>
+        <v>8.136428466540477e-14</v>
       </c>
     </row>
     <row r="51">
@@ -3217,52 +3217,52 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>6.237378877304954e-07</v>
+        <v>1.06592233679514e-07</v>
       </c>
       <c r="C51" t="n">
-        <v>0.002878999999999939</v>
+        <v>0.0004919999999998569</v>
       </c>
       <c r="D51" t="n">
-        <v>0.01107482842173374</v>
+        <v>0.001892607010591014</v>
       </c>
       <c r="E51" t="n">
-        <v>3.685204759083829e-09</v>
+        <v>6.297744847060629e-10</v>
       </c>
       <c r="F51" t="n">
-        <v>1.879420933233865e-07</v>
+        <v>3.211792633382466e-08</v>
       </c>
       <c r="G51" t="n">
-        <v>1.473853064872751e-06</v>
+        <v>2.518706870153518e-07</v>
       </c>
       <c r="H51" t="n">
-        <v>5.772771611603304e-14</v>
+        <v>9.865243601625771e-15</v>
       </c>
       <c r="I51" t="n">
-        <v>1.873134832632169e-12</v>
+        <v>3.201050148158314e-13</v>
       </c>
       <c r="J51" t="n">
-        <v>3.76576752353176e-06</v>
+        <v>6.435420707110546e-07</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0007469098344928762</v>
+        <v>0.000127641416662173</v>
       </c>
       <c r="L51" t="n">
-        <v>1.641568649544594e-10</v>
+        <v>2.805320512593687e-11</v>
       </c>
       <c r="M51" t="n">
-        <v>4.83686547031924e-12</v>
+        <v>8.265848598111929e-13</v>
       </c>
       <c r="N51" t="n">
-        <v>5.934086614498193e-07</v>
+        <v>1.014091911890352e-07</v>
       </c>
       <c r="O51" t="n">
-        <v>2.460195387161219e-05</v>
+        <v>4.204293610569619e-06</v>
       </c>
       <c r="P51" t="n">
-        <v>0.0007303375485991564</v>
+        <v>0.0001248093344601209</v>
       </c>
       <c r="Q51" t="n">
-        <v>1.113994446999339e-11</v>
+        <v>1.903734866007388e-12</v>
       </c>
     </row>
     <row r="52">
@@ -3272,52 +3272,52 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>6.677639239649407e-07</v>
+        <v>1.399576252714714e-07</v>
       </c>
       <c r="C52" t="n">
-        <v>0.0005629999999999425</v>
+        <v>0.0001179999999999511</v>
       </c>
       <c r="D52" t="n">
-        <v>0.007209363888098399</v>
+        <v>0.001511021205675569</v>
       </c>
       <c r="E52" t="n">
-        <v>8.879990674837612e-10</v>
+        <v>1.861170336821511e-10</v>
       </c>
       <c r="F52" t="n">
-        <v>1.90550017762028e-07</v>
+        <v>3.993765914016391e-08</v>
       </c>
       <c r="G52" t="n">
-        <v>3.330915802323042e-06</v>
+        <v>6.981315535950198e-07</v>
       </c>
       <c r="H52" t="n">
-        <v>6.471368904667316e-14</v>
+        <v>1.356343749112797e-14</v>
       </c>
       <c r="I52" t="n">
-        <v>2.703950946340839e-12</v>
+        <v>5.667250651298744e-13</v>
       </c>
       <c r="J52" t="n">
-        <v>2.694631217565001e-08</v>
+        <v>5.647717294361826e-09</v>
       </c>
       <c r="K52" t="n">
-        <v>6.042126027315621e-06</v>
+        <v>1.266378101639468e-06</v>
       </c>
       <c r="L52" t="n">
-        <v>6.302274764826274e-12</v>
+        <v>1.320903059057314e-12</v>
       </c>
       <c r="M52" t="n">
-        <v>9.22828197193182e-12</v>
+        <v>1.934169223246207e-12</v>
       </c>
       <c r="N52" t="n">
-        <v>4.902913622607105e-07</v>
+        <v>1.027608894258361e-07</v>
       </c>
       <c r="O52" t="n">
-        <v>1.513675638305976e-05</v>
+        <v>3.172535085613665e-06</v>
       </c>
       <c r="P52" t="n">
-        <v>9.575021959702578e-06</v>
+        <v>2.006842968462791e-06</v>
       </c>
       <c r="Q52" t="n">
-        <v>6.238130907474848e-14</v>
+        <v>1.307459053431265e-14</v>
       </c>
     </row>
     <row r="53">
@@ -3382,52 +3382,52 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.01244566297376408</v>
+        <v>0.01404447300937334</v>
       </c>
       <c r="C54" t="n">
-        <v>394.156989</v>
+        <v>444.791668</v>
       </c>
       <c r="D54" t="n">
-        <v>66.82332350486354</v>
+        <v>75.40766332328528</v>
       </c>
       <c r="E54" t="n">
-        <v>0.0002179130304246816</v>
+        <v>0.0002459068416557467</v>
       </c>
       <c r="F54" t="n">
-        <v>0.001572472897481475</v>
+        <v>0.001774477841253193</v>
       </c>
       <c r="G54" t="n">
-        <v>0.01641189940341527</v>
+        <v>0.0185202249723226</v>
       </c>
       <c r="H54" t="n">
-        <v>8.775248096906373e-09</v>
+        <v>9.902544790692044e-09</v>
       </c>
       <c r="I54" t="n">
-        <v>8.602996669525243e-08</v>
+        <v>9.7081653889856e-08</v>
       </c>
       <c r="J54" t="n">
-        <v>0.108419279852294</v>
+        <v>0.1223471704794778</v>
       </c>
       <c r="K54" t="n">
-        <v>8.309164769089524</v>
+        <v>9.37658689423915</v>
       </c>
       <c r="L54" t="n">
-        <v>7.740788143539098e-05</v>
+        <v>8.73519477286087e-05</v>
       </c>
       <c r="M54" t="n">
-        <v>1.735748669422273e-07</v>
+        <v>1.958728545851342e-07</v>
       </c>
       <c r="N54" t="n">
-        <v>0.008999619916340046</v>
+        <v>0.01015574013823946</v>
       </c>
       <c r="O54" t="n">
-        <v>1.510892052232176</v>
+        <v>1.704986121862964</v>
       </c>
       <c r="P54" t="n">
-        <v>19.29082412199759</v>
+        <v>21.7689856523588</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.000235322207627276</v>
+        <v>0.0002655524579521751</v>
       </c>
     </row>
     <row r="55">
@@ -3602,52 +3602,52 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1.616748591310807e-07</v>
+        <v>3.058713551128842e-08</v>
       </c>
       <c r="C58" t="n">
-        <v>0.0002959999999999682</v>
+        <v>5.599999999999925e-05</v>
       </c>
       <c r="D58" t="n">
-        <v>0.007161483845085552</v>
+        <v>0.00135487532204334</v>
       </c>
       <c r="E58" t="n">
-        <v>2.560628721930669e-09</v>
+        <v>4.844432717166586e-10</v>
       </c>
       <c r="F58" t="n">
-        <v>9.45729641708444e-08</v>
+        <v>1.789218241070197e-08</v>
       </c>
       <c r="G58" t="n">
-        <v>7.45726838778671e-07</v>
+        <v>1.410834559851672e-07</v>
       </c>
       <c r="H58" t="n">
-        <v>2.602367833092522e-14</v>
+        <v>4.923398603148478e-15</v>
       </c>
       <c r="I58" t="n">
-        <v>1.967626119562865e-12</v>
+        <v>3.722535901876041e-13</v>
       </c>
       <c r="J58" t="n">
-        <v>3.574103918856273e-07</v>
+        <v>6.761818224863856e-08</v>
       </c>
       <c r="K58" t="n">
-        <v>0.000359482589310777</v>
+        <v>6.80102195993426e-05</v>
       </c>
       <c r="L58" t="n">
-        <v>2.693356334466834e-10</v>
+        <v>5.095539011153948e-11</v>
       </c>
       <c r="M58" t="n">
-        <v>1.701191278621237e-12</v>
+        <v>3.218469986581021e-13</v>
       </c>
       <c r="N58" t="n">
-        <v>1.546151528024607e-07</v>
+        <v>2.925151539506289e-08</v>
       </c>
       <c r="O58" t="n">
-        <v>2.017659885715757e-05</v>
+        <v>3.817194378381522e-06</v>
       </c>
       <c r="P58" t="n">
-        <v>5.454303705321725e-05</v>
+        <v>1.031895295601504e-05</v>
       </c>
       <c r="Q58" t="n">
-        <v>1.073673295974597e-12</v>
+        <v>2.031273803195374e-13</v>
       </c>
     </row>
     <row r="59">
@@ -3770,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>0.001020999999999984</v>
+        <v>5.199999999998937e-05</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -3932,52 +3932,52 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.01727259708563632</v>
+        <v>0.01727280762368704</v>
       </c>
       <c r="C64" t="n">
-        <v>1.558765</v>
+        <v>1.558784</v>
       </c>
       <c r="D64" t="n">
-        <v>4785.552888581158</v>
+        <v>4785.611220340521</v>
       </c>
       <c r="E64" t="n">
-        <v>0.002060337666963863</v>
+        <v>0.002060362780701772</v>
       </c>
       <c r="F64" t="n">
-        <v>0.04157971220296563</v>
+        <v>0.04158021902377047</v>
       </c>
       <c r="G64" t="n">
-        <v>0.03368777608140298</v>
+        <v>0.03368818670631793</v>
       </c>
       <c r="H64" t="n">
-        <v>8.516944741146639e-09</v>
+        <v>8.517048555352169e-09</v>
       </c>
       <c r="I64" t="n">
-        <v>2.386232021736292e-07</v>
+        <v>2.386261107845111e-07</v>
       </c>
       <c r="J64" t="n">
-        <v>0.1280252612794011</v>
+        <v>0.1280268217968391</v>
       </c>
       <c r="K64" t="n">
-        <v>24.05906788999517</v>
+        <v>24.05936114926767</v>
       </c>
       <c r="L64" t="n">
-        <v>4.495891799379137e-05</v>
+        <v>4.495946600419825e-05</v>
       </c>
       <c r="M64" t="n">
-        <v>2.580888952203571e-07</v>
+        <v>2.580920411012366e-07</v>
       </c>
       <c r="N64" t="n">
-        <v>0.005592897423695045</v>
+        <v>0.005592965596287482</v>
       </c>
       <c r="O64" t="n">
-        <v>12.15326792877133</v>
+        <v>12.15341606661806</v>
       </c>
       <c r="P64" t="n">
-        <v>13.60041800157931</v>
+        <v>13.6005837789364</v>
       </c>
       <c r="Q64" t="n">
-        <v>6.581689369045264e-07</v>
+        <v>6.581769594158101e-07</v>
       </c>
     </row>
     <row r="65">
@@ -4097,52 +4097,52 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1.815942962740096e-06</v>
+        <v>6.053143209133506e-07</v>
       </c>
       <c r="C67" t="n">
-        <v>8.999999999999953e-06</v>
+        <v>2.999999999999911e-06</v>
       </c>
       <c r="D67" t="n">
-        <v>0.001199406620836261</v>
+        <v>0.0003998022069454106</v>
       </c>
       <c r="E67" t="n">
-        <v>6.851383151160461e-09</v>
+        <v>2.283794383720097e-09</v>
       </c>
       <c r="F67" t="n">
-        <v>6.112636006223618e-07</v>
+        <v>2.037545335407822e-07</v>
       </c>
       <c r="G67" t="n">
-        <v>4.681875844105948e-06</v>
+        <v>1.560625281368611e-06</v>
       </c>
       <c r="H67" t="n">
-        <v>1.018703244949716e-13</v>
+        <v>3.395677483165638e-14</v>
       </c>
       <c r="I67" t="n">
-        <v>4.284007601937915e-13</v>
+        <v>1.42800253397927e-13</v>
       </c>
       <c r="J67" t="n">
-        <v>2.17719932988716e-06</v>
+        <v>7.257331099623687e-07</v>
       </c>
       <c r="K67" t="n">
-        <v>9.069563349368551e-05</v>
+        <v>3.023187783122776e-05</v>
       </c>
       <c r="L67" t="n">
-        <v>1.220063269365088e-09</v>
+        <v>4.066877564550193e-10</v>
       </c>
       <c r="M67" t="n">
-        <v>3.502228728723204e-12</v>
+        <v>1.167409576241039e-12</v>
       </c>
       <c r="N67" t="n">
-        <v>1.17433809001661e-06</v>
+        <v>3.914460300055269e-07</v>
       </c>
       <c r="O67" t="n">
-        <v>0.003572363996792886</v>
+        <v>0.001190787998930933</v>
       </c>
       <c r="P67" t="n">
-        <v>0.0001170371128803392</v>
+        <v>3.901237096011211e-05</v>
       </c>
       <c r="Q67" t="n">
-        <v>8.419365257869931e-13</v>
+        <v>2.806455085956575e-13</v>
       </c>
     </row>
     <row r="68">
@@ -4152,52 +4152,52 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>6.59831591049844e-05</v>
+        <v>6.616093756474912e-05</v>
       </c>
       <c r="C68" t="n">
-        <v>0.009650000000000001</v>
+        <v>0.009676000000000001</v>
       </c>
       <c r="D68" t="n">
-        <v>0.3469269649439196</v>
+        <v>0.3478616904453228</v>
       </c>
       <c r="E68" t="n">
-        <v>1.494095006880112e-06</v>
+        <v>1.498120547831292e-06</v>
       </c>
       <c r="F68" t="n">
-        <v>3.767212298150358e-05</v>
+        <v>3.777362300197188e-05</v>
       </c>
       <c r="G68" t="n">
-        <v>0.0002052353006651649</v>
+        <v>0.0002057882662420866</v>
       </c>
       <c r="H68" t="n">
-        <v>6.933597232007871e-12</v>
+        <v>6.952278426622606e-12</v>
       </c>
       <c r="I68" t="n">
-        <v>2.172428994284353e-10</v>
+        <v>2.178282170849264e-10</v>
       </c>
       <c r="J68" t="n">
-        <v>0.001071199519591363</v>
+        <v>0.001074085653012024</v>
       </c>
       <c r="K68" t="n">
-        <v>-8.899457763225945</v>
+        <v>-8.923435576888521</v>
       </c>
       <c r="L68" t="n">
-        <v>1.304547918831258e-07</v>
+        <v>1.308062762964896e-07</v>
       </c>
       <c r="M68" t="n">
-        <v>5.97578373029247e-10</v>
+        <v>5.991884287493257e-10</v>
       </c>
       <c r="N68" t="n">
-        <v>0.0001079885277537337</v>
+        <v>0.0001082794813000132</v>
       </c>
       <c r="O68" t="n">
-        <v>0.02057680133469665</v>
+        <v>0.02063224142119428</v>
       </c>
       <c r="P68" t="n">
-        <v>0.2042390410326602</v>
+        <v>0.2047893223867378</v>
       </c>
       <c r="Q68" t="n">
-        <v>2.604560109427166e-09</v>
+        <v>2.611577577079509e-09</v>
       </c>
     </row>
     <row r="69">
@@ -4207,52 +4207,52 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>6.111300025783377e-08</v>
+        <v>9.25954549361227e-09</v>
       </c>
       <c r="C69" t="n">
-        <v>3.299999999999611e-05</v>
+        <v>5e-06</v>
       </c>
       <c r="D69" t="n">
-        <v>3.588698040310916e-05</v>
+        <v>5.437421273199e-06</v>
       </c>
       <c r="E69" t="n">
-        <v>2.268056495473989e-10</v>
+        <v>3.436449235567056e-11</v>
       </c>
       <c r="F69" t="n">
-        <v>9.430726080410507e-09</v>
+        <v>1.428897890971458e-09</v>
       </c>
       <c r="G69" t="n">
-        <v>2.578097715870237e-07</v>
+        <v>3.90620866040991e-08</v>
       </c>
       <c r="H69" t="n">
-        <v>6.296150941459084e-15</v>
+        <v>9.539622638575496e-16</v>
       </c>
       <c r="I69" t="n">
-        <v>2.054443653652858e-14</v>
+        <v>3.112793414625909e-15</v>
       </c>
       <c r="J69" t="n">
-        <v>9.298921496296387e-08</v>
+        <v>1.408927499439013e-08</v>
       </c>
       <c r="K69" t="n">
-        <v>6.37627410062417e-06</v>
+        <v>9.661021364583218e-07</v>
       </c>
       <c r="L69" t="n">
-        <v>2.338440411067047e-11</v>
+        <v>3.543091531920187e-12</v>
       </c>
       <c r="M69" t="n">
-        <v>4.51800436008853e-13</v>
+        <v>6.845461151650096e-14</v>
       </c>
       <c r="N69" t="n">
-        <v>4.829231396429407e-09</v>
+        <v>7.317017267318147e-10</v>
       </c>
       <c r="O69" t="n">
-        <v>1.170556818117631e-06</v>
+        <v>1.773570936542075e-07</v>
       </c>
       <c r="P69" t="n">
-        <v>4.081574376024515e-05</v>
+        <v>6.184203600037875e-06</v>
       </c>
       <c r="Q69" t="n">
-        <v>9.094231998715568e-14</v>
+        <v>1.377913939199491e-14</v>
       </c>
     </row>
     <row r="70">
@@ -4262,52 +4262,52 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>63.6234702116226</v>
+        <v>60.47696147917164</v>
       </c>
       <c r="C70" t="n">
-        <v>7326.224972</v>
+        <v>6963.905362999999</v>
       </c>
       <c r="D70" t="n">
-        <v>163171.5873791627</v>
+        <v>155101.9108451935</v>
       </c>
       <c r="E70" t="n">
-        <v>0.0373966265911299</v>
+        <v>0.03554717053754131</v>
       </c>
       <c r="F70" t="n">
-        <v>6.169697820574131</v>
+        <v>5.864574443863473</v>
       </c>
       <c r="G70" t="n">
-        <v>67.55235525614785</v>
+        <v>64.21154289548743</v>
       </c>
       <c r="H70" t="n">
-        <v>1.136767065650701e-06</v>
+        <v>1.080548071513232e-06</v>
       </c>
       <c r="I70" t="n">
-        <v>7.010363003297397e-05</v>
+        <v>6.663664397670305e-05</v>
       </c>
       <c r="J70" t="n">
-        <v>1.407099856583803</v>
+        <v>1.337511511725451</v>
       </c>
       <c r="K70" t="n">
-        <v>243.2130029225717</v>
+        <v>231.1848655858928</v>
       </c>
       <c r="L70" t="n">
-        <v>5.663091066594092e-05</v>
+        <v>5.383022006631874e-05</v>
       </c>
       <c r="M70" t="n">
-        <v>0.000807425394389048</v>
+        <v>0.0007674940444359973</v>
       </c>
       <c r="N70" t="n">
-        <v>20.13646478026329</v>
+        <v>19.1406127454553</v>
       </c>
       <c r="O70" t="n">
-        <v>5.852149128346503</v>
+        <v>5.562730172186143</v>
       </c>
       <c r="P70" t="n">
-        <v>59.1599839173205</v>
+        <v>56.23421760202287</v>
       </c>
       <c r="Q70" t="n">
-        <v>9.900378840949886e-07</v>
+        <v>9.410754047237663e-07</v>
       </c>
     </row>
     <row r="71">
@@ -4317,28 +4317,28 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.7129690559295915</v>
+        <v>0.7493367053720945</v>
       </c>
       <c r="C71" t="n">
-        <v>2256.308857999999</v>
+        <v>2371.400318</v>
       </c>
       <c r="D71" t="n">
-        <v>1.978061110879441</v>
+        <v>2.078959505358171</v>
       </c>
       <c r="E71" t="n">
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>0.359569011954647</v>
+        <v>0.3779101723015066</v>
       </c>
       <c r="G71" t="n">
-        <v>3.937696860818849</v>
+        <v>4.138553795427869</v>
       </c>
       <c r="H71" t="n">
-        <v>1.115491362710846e-07</v>
+        <v>1.172391165721672e-07</v>
       </c>
       <c r="I71" t="n">
-        <v>7.786599391704523e-07</v>
+        <v>8.183783974501736e-07</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
@@ -4350,10 +4350,10 @@
         <v>0</v>
       </c>
       <c r="M71" t="n">
-        <v>2.614268118410117e-06</v>
+        <v>2.747618627367465e-06</v>
       </c>
       <c r="N71" t="n">
-        <v>1.023252353479495</v>
+        <v>1.075447161336953</v>
       </c>
       <c r="O71" t="n">
         <v>0</v>
@@ -4372,28 +4372,28 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>8.216158616004928e-07</v>
+        <v>1.504742177647338e-07</v>
       </c>
       <c r="C72" t="n">
-        <v>0.000616999999999988</v>
+        <v>0.0001129999999999796</v>
       </c>
       <c r="D72" t="n">
-        <v>0.0002159721352458868</v>
+        <v>3.955405394291942e-05</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>1.618380360267529e-07</v>
+        <v>2.963970513941675e-08</v>
       </c>
       <c r="G72" t="n">
-        <v>1.78785732528969e-06</v>
+        <v>3.274357824273946e-07</v>
       </c>
       <c r="H72" t="n">
-        <v>1.943399500451616e-13</v>
+        <v>3.559224368735773e-14</v>
       </c>
       <c r="I72" t="n">
-        <v>8.926515306555978e-13</v>
+        <v>1.634839918380329e-13</v>
       </c>
       <c r="J72" t="n">
         <v>0</v>
@@ -4405,10 +4405,10 @@
         <v>0</v>
       </c>
       <c r="M72" t="n">
-        <v>3.996683258541004e-12</v>
+        <v>7.319695432983157e-13</v>
       </c>
       <c r="N72" t="n">
-        <v>4.5857831825853e-07</v>
+        <v>8.398598049141904e-08</v>
       </c>
       <c r="O72" t="n">
         <v>0</v>
@@ -4427,52 +4427,52 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1.030070751046104</v>
+        <v>1.030070967943164</v>
       </c>
       <c r="C73" t="n">
-        <v>4896.345498</v>
+        <v>4896.346529</v>
       </c>
       <c r="D73" t="n">
-        <v>10674.63478539175</v>
+        <v>10674.63703309843</v>
       </c>
       <c r="E73" t="n">
-        <v>0.008241792795564773</v>
+        <v>0.008241794530999576</v>
       </c>
       <c r="F73" t="n">
-        <v>0.613446193401765</v>
+        <v>0.6134463225721893</v>
       </c>
       <c r="G73" t="n">
-        <v>5.160782961993764</v>
+        <v>5.160784048675095</v>
       </c>
       <c r="H73" t="n">
-        <v>2.510138450915118e-07</v>
+        <v>2.510138979462939e-07</v>
       </c>
       <c r="I73" t="n">
-        <v>1.32623107810855e-05</v>
+        <v>1.32623135736667e-05</v>
       </c>
       <c r="J73" t="n">
-        <v>2.769638469409537</v>
+        <v>2.769639052599033</v>
       </c>
       <c r="K73" t="n">
-        <v>170.7825002161667</v>
+        <v>170.7825361770191</v>
       </c>
       <c r="L73" t="n">
-        <v>0.00032188254784359</v>
+        <v>0.0003218826156208551</v>
       </c>
       <c r="M73" t="n">
-        <v>3.918606792823044e-06</v>
+        <v>3.918607617945293e-06</v>
       </c>
       <c r="N73" t="n">
-        <v>1.225947258410931</v>
+        <v>1.225947516552769</v>
       </c>
       <c r="O73" t="n">
-        <v>330.5449724682281</v>
+        <v>330.5450420694985</v>
       </c>
       <c r="P73" t="n">
-        <v>407.4424070057131</v>
+        <v>407.4424927989076</v>
       </c>
       <c r="Q73" t="n">
-        <v>7.661300940758563e-06</v>
+        <v>7.661302553961978e-06</v>
       </c>
     </row>
     <row r="74">
@@ -4482,52 +4482,52 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>3.024362868511634e-06</v>
+        <v>6.774195957818751e-07</v>
       </c>
       <c r="C74" t="n">
-        <v>0.00321</v>
+        <v>0.0007189999999999848</v>
       </c>
       <c r="D74" t="n">
-        <v>0.04397152585727467</v>
+        <v>0.009849073860242934</v>
       </c>
       <c r="E74" t="n">
-        <v>4.597605179426096e-09</v>
+        <v>1.02980626916115e-09</v>
       </c>
       <c r="F74" t="n">
-        <v>1.455812620897094e-06</v>
+        <v>3.260838861137036e-07</v>
       </c>
       <c r="G74" t="n">
-        <v>1.661179835264529e-05</v>
+        <v>3.720835830389942e-06</v>
       </c>
       <c r="H74" t="n">
-        <v>3.567817238740415e-13</v>
+        <v>7.991466026960449e-14</v>
       </c>
       <c r="I74" t="n">
-        <v>2.049189828124239e-11</v>
+        <v>4.5899298642408e-12</v>
       </c>
       <c r="J74" t="n">
-        <v>1.389049827552516e-08</v>
+        <v>3.11129852339638e-09</v>
       </c>
       <c r="K74" t="n">
-        <v>6.899917344011674e-06</v>
+        <v>1.545495504780152e-06</v>
       </c>
       <c r="L74" t="n">
-        <v>3.540101374906539e-12</v>
+        <v>7.929385945662765e-13</v>
       </c>
       <c r="M74" t="n">
-        <v>7.493278836874346e-11</v>
+        <v>1.678401085268704e-11</v>
       </c>
       <c r="N74" t="n">
-        <v>3.94484849246745e-06</v>
+        <v>8.835969053221298e-07</v>
       </c>
       <c r="O74" t="n">
-        <v>0.0001068961807135855</v>
+        <v>2.394341244020759e-05</v>
       </c>
       <c r="P74" t="n">
-        <v>2.524911679165117e-06</v>
+        <v>5.655487530590906e-07</v>
       </c>
       <c r="Q74" t="n">
-        <v>3.725235901918918e-14</v>
+        <v>8.344064216447494e-15</v>
       </c>
     </row>
     <row r="75">
@@ -4537,52 +4537,52 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>7.437326840187078</v>
+        <v>9.365533395439039</v>
       </c>
       <c r="C75" t="n">
-        <v>8480.148504999999</v>
+        <v>10678.717734</v>
       </c>
       <c r="D75" t="n">
-        <v>367.7699270598205</v>
+        <v>463.118215419223</v>
       </c>
       <c r="E75" t="n">
-        <v>0.001567596753339762</v>
+        <v>0.001974012983355194</v>
       </c>
       <c r="F75" t="n">
-        <v>3.859478231906161</v>
+        <v>4.860089256071735</v>
       </c>
       <c r="G75" t="n">
-        <v>42.05657606789735</v>
+        <v>52.96019337665778</v>
       </c>
       <c r="H75" t="n">
-        <v>7.078161621150548e-09</v>
+        <v>8.913250750659883e-09</v>
       </c>
       <c r="I75" t="n">
-        <v>2.470663399960249e-05</v>
+        <v>3.111209320018888e-05</v>
       </c>
       <c r="J75" t="n">
-        <v>1.082076712603577</v>
+        <v>1.362616677480961</v>
       </c>
       <c r="K75" t="n">
-        <v>514.4092441062496</v>
+        <v>647.7753443034713</v>
       </c>
       <c r="L75" t="n">
-        <v>0.0001317559186721156</v>
+        <v>0.0001659150502439676</v>
       </c>
       <c r="M75" t="n">
-        <v>2.196300293725139e-05</v>
+        <v>2.765714643082427e-05</v>
       </c>
       <c r="N75" t="n">
-        <v>12.4797558714317</v>
+        <v>15.71526610196414</v>
       </c>
       <c r="O75" t="n">
-        <v>20.77996805200571</v>
+        <v>26.16739709429261</v>
       </c>
       <c r="P75" t="n">
-        <v>206.0635104444338</v>
+        <v>259.48768019992</v>
       </c>
       <c r="Q75" t="n">
-        <v>2.628166793404458e-06</v>
+        <v>3.309547153341756e-06</v>
       </c>
     </row>
     <row r="76">
@@ -4592,52 +4592,52 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>8.141528836509369e-08</v>
+        <v>1.388477786071518e-08</v>
       </c>
       <c r="C76" t="n">
-        <v>0.0003869999999999576</v>
+        <v>6.600000000000001e-05</v>
       </c>
       <c r="D76" t="n">
-        <v>0.0008437075495660117</v>
+        <v>0.0001438881092283279</v>
       </c>
       <c r="E76" t="n">
-        <v>6.514192703897329e-10</v>
+        <v>1.110947592912845e-10</v>
       </c>
       <c r="F76" t="n">
-        <v>4.84858915579852e-08</v>
+        <v>8.268911738572027e-09</v>
       </c>
       <c r="G76" t="n">
-        <v>4.079007511024641e-07</v>
+        <v>6.956446918027283e-08</v>
       </c>
       <c r="H76" t="n">
-        <v>1.983976786157838e-14</v>
+        <v>3.383526301974978e-15</v>
       </c>
       <c r="I76" t="n">
-        <v>1.04823368252424e-12</v>
+        <v>1.787685350041535e-13</v>
       </c>
       <c r="J76" t="n">
-        <v>2.189081812341824e-07</v>
+        <v>3.733317819498095e-08</v>
       </c>
       <c r="K76" t="n">
-        <v>1.349839949216125e-05</v>
+        <v>2.302052626570388e-06</v>
       </c>
       <c r="L76" t="n">
-        <v>2.544112666606904e-11</v>
+        <v>4.338796795764187e-12</v>
       </c>
       <c r="M76" t="n">
-        <v>3.097209601409445e-13</v>
+        <v>5.282062886125215e-14</v>
       </c>
       <c r="N76" t="n">
-        <v>9.689708154760984e-08</v>
+        <v>1.652508367478799e-08</v>
       </c>
       <c r="O76" t="n">
-        <v>2.612579206214959e-05</v>
+        <v>4.455561436956232e-06</v>
       </c>
       <c r="P76" t="n">
-        <v>3.220365302562912e-05</v>
+        <v>5.492095864836576e-06</v>
       </c>
       <c r="Q76" t="n">
-        <v>6.055380416443885e-13</v>
+        <v>1.03270053613783e-13</v>
       </c>
     </row>
     <row r="77">
@@ -4647,52 +4647,52 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>6.677117557369314e-06</v>
+        <v>1.183659677326951e-06</v>
       </c>
       <c r="C77" t="n">
-        <v>0.005437999999999998</v>
+        <v>0.0009639999999999911</v>
       </c>
       <c r="D77" t="n">
-        <v>0.08777577547895168</v>
+        <v>0.01556010436956761</v>
       </c>
       <c r="E77" t="n">
-        <v>9.421111929969724e-09</v>
+        <v>1.67009045614026e-09</v>
       </c>
       <c r="F77" t="n">
-        <v>3.268622365042851e-06</v>
+        <v>5.794321367968519e-07</v>
       </c>
       <c r="G77" t="n">
-        <v>3.698042495399067e-05</v>
+        <v>6.555558965731278e-06</v>
       </c>
       <c r="H77" t="n">
-        <v>6.634905800030361e-13</v>
+        <v>1.176176754547483e-13</v>
       </c>
       <c r="I77" t="n">
-        <v>4.14563146332552e-11</v>
+        <v>7.34900465363326e-12</v>
       </c>
       <c r="J77" t="n">
-        <v>1.146577189119198e-07</v>
+        <v>2.03254948567653e-08</v>
       </c>
       <c r="K77" t="n">
-        <v>4.278512422610019e-05</v>
+        <v>7.584564132762086e-06</v>
       </c>
       <c r="L77" t="n">
-        <v>2.920857075274475e-11</v>
+        <v>5.177834168011345e-12</v>
       </c>
       <c r="M77" t="n">
-        <v>6.224122319577559e-10</v>
+        <v>1.103356733371224e-10</v>
       </c>
       <c r="N77" t="n">
-        <v>8.843265843719817e-06</v>
+        <v>1.5676550704939e-06</v>
       </c>
       <c r="O77" t="n">
-        <v>0.0001413791073230899</v>
+        <v>2.50624235857774e-05</v>
       </c>
       <c r="P77" t="n">
-        <v>3.611440556602912e-05</v>
+        <v>6.402038794713455e-06</v>
       </c>
       <c r="Q77" t="n">
-        <v>2.899783983224405e-13</v>
+        <v>5.140477675300298e-14</v>
       </c>
     </row>
     <row r="78">
@@ -4812,52 +4812,52 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>3.567871628844729e-08</v>
+        <v>7.135743257687108e-09</v>
       </c>
       <c r="C80" t="n">
-        <v>4.999999999999616e-06</v>
+        <v>9.999999999995938e-07</v>
       </c>
       <c r="D80" t="n">
-        <v>0.0003753135312854213</v>
+        <v>7.506270625705954e-05</v>
       </c>
       <c r="E80" t="n">
-        <v>2.46547036054644e-09</v>
+        <v>4.930940721091256e-10</v>
       </c>
       <c r="F80" t="n">
-        <v>1.029591041070367e-08</v>
+        <v>2.059182082140055e-09</v>
       </c>
       <c r="G80" t="n">
-        <v>1.140782874166793e-07</v>
+        <v>2.281565748332834e-08</v>
       </c>
       <c r="H80" t="n">
-        <v>3.274936187854484e-15</v>
+        <v>6.54987237570681e-16</v>
       </c>
       <c r="I80" t="n">
-        <v>1.100422601953662e-13</v>
+        <v>2.2008452039066e-14</v>
       </c>
       <c r="J80" t="n">
-        <v>3.050116091337361e-08</v>
+        <v>6.100232182672713e-09</v>
       </c>
       <c r="K80" t="n">
-        <v>5.089588711235162e-06</v>
+        <v>1.017917742246697e-06</v>
       </c>
       <c r="L80" t="n">
-        <v>3.084067704883819e-10</v>
+        <v>6.168135409765606e-11</v>
       </c>
       <c r="M80" t="n">
-        <v>4.686367089488558e-14</v>
+        <v>9.372734178974028e-15</v>
       </c>
       <c r="N80" t="n">
-        <v>4.99165920217315e-08</v>
+        <v>9.983318404343011e-09</v>
       </c>
       <c r="O80" t="n">
-        <v>2.428841836455815e-05</v>
+        <v>4.857683672910031e-06</v>
       </c>
       <c r="P80" t="n">
-        <v>2.288587324959045e-06</v>
+        <v>4.577174649916583e-07</v>
       </c>
       <c r="Q80" t="n">
-        <v>4.739417871232229e-14</v>
+        <v>9.478835742461335e-15</v>
       </c>
     </row>
     <row r="81">
@@ -5035,7 +5035,7 @@
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>0.001279999999999982</v>
+        <v>8.39999999999878e-05</v>
       </c>
       <c r="D84" t="n">
         <v>0</v>
@@ -5252,52 +5252,52 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>9.026217511702609e-08</v>
+        <v>9.872425403428241e-09</v>
       </c>
       <c r="C88" t="n">
-        <v>0.0002559999999999089</v>
+        <v>2.8e-05</v>
       </c>
       <c r="D88" t="n">
-        <v>0.004056411750366726</v>
+        <v>0.0004436700351965185</v>
       </c>
       <c r="E88" t="n">
-        <v>2.216227941664449e-09</v>
+        <v>2.423999311196353e-10</v>
       </c>
       <c r="F88" t="n">
-        <v>1.417030515999518e-08</v>
+        <v>1.549877126875024e-09</v>
       </c>
       <c r="G88" t="n">
-        <v>1.417813115886662e-07</v>
+        <v>1.550733095501588e-08</v>
       </c>
       <c r="H88" t="n">
-        <v>6.331620362287899e-15</v>
+        <v>6.925209771254854e-16</v>
       </c>
       <c r="I88" t="n">
-        <v>1.633583677371401e-13</v>
+        <v>1.786732147125605e-14</v>
       </c>
       <c r="J88" t="n">
-        <v>2.477567081406543e-06</v>
+        <v>2.709838995289371e-07</v>
       </c>
       <c r="K88" t="n">
-        <v>0.000101591096231349</v>
+        <v>1.111152615030775e-05</v>
       </c>
       <c r="L88" t="n">
-        <v>2.041483142915052e-10</v>
+        <v>2.232872187564133e-11</v>
       </c>
       <c r="M88" t="n">
-        <v>6.539974298851525e-13</v>
+        <v>7.1530968893714e-14</v>
       </c>
       <c r="N88" t="n">
-        <v>3.403520729779801e-08</v>
+        <v>3.722600798197982e-09</v>
       </c>
       <c r="O88" t="n">
-        <v>3.274997128482395e-05</v>
+        <v>3.582028109278894e-06</v>
       </c>
       <c r="P88" t="n">
-        <v>8.459252447058332e-05</v>
+        <v>9.252307363973343e-06</v>
       </c>
       <c r="Q88" t="n">
-        <v>6.878004324297762e-13</v>
+        <v>7.522817229703354e-14</v>
       </c>
     </row>
     <row r="89">
@@ -5307,52 +5307,52 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>3.087096175238127e-06</v>
+        <v>1.50403242100244e-07</v>
       </c>
       <c r="C89" t="n">
-        <v>0.02660099999999998</v>
+        <v>0.001295999999999992</v>
       </c>
       <c r="D89" t="n">
-        <v>0.04616799190820989</v>
+        <v>0.00224930331615502</v>
       </c>
       <c r="E89" t="n">
-        <v>5.543661092099004e-08</v>
+        <v>2.700870183587185e-09</v>
       </c>
       <c r="F89" t="n">
-        <v>7.036844448128309e-07</v>
+        <v>3.42834871048992e-08</v>
       </c>
       <c r="G89" t="n">
-        <v>7.73878867489404e-06</v>
+        <v>3.770335747777384e-07</v>
       </c>
       <c r="H89" t="n">
-        <v>4.329811482159281e-13</v>
+        <v>2.109482982173e-14</v>
       </c>
       <c r="I89" t="n">
-        <v>8.72069185403697e-12</v>
+        <v>4.248718710887504e-13</v>
       </c>
       <c r="J89" t="n">
-        <v>4.978688331280836e-06</v>
+        <v>2.425615607435784e-07</v>
       </c>
       <c r="K89" t="n">
-        <v>0.0004499117924142579</v>
+        <v>2.191969034881678e-05</v>
       </c>
       <c r="L89" t="n">
-        <v>1.615693625978395e-08</v>
+        <v>7.871654972625047e-10</v>
       </c>
       <c r="M89" t="n">
-        <v>1.236046422877929e-11</v>
+        <v>6.022014826697443e-13</v>
       </c>
       <c r="N89" t="n">
-        <v>2.100907667939168e-06</v>
+        <v>1.023561647174598e-07</v>
       </c>
       <c r="O89" t="n">
-        <v>0.001253704262007955</v>
+        <v>6.108043771145072e-05</v>
       </c>
       <c r="P89" t="n">
-        <v>0.0004379332706692459</v>
+        <v>2.133609709361827e-05</v>
       </c>
       <c r="Q89" t="n">
-        <v>1.030401248339529e-11</v>
+        <v>5.020112092958995e-13</v>
       </c>
     </row>
     <row r="90">
@@ -5417,52 +5417,52 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2.7795715443373e-08</v>
+        <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>2.999999999999886e-06</v>
+        <v>0</v>
       </c>
       <c r="D91" t="n">
-        <v>0.001964601334187335</v>
+        <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>5.038945928210884e-09</v>
+        <v>0</v>
       </c>
       <c r="F91" t="n">
-        <v>1.018707081059073e-07</v>
+        <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>7.981089517229384e-08</v>
+        <v>0</v>
       </c>
       <c r="H91" t="n">
-        <v>2.470628349575555e-14</v>
+        <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>5.780338501111965e-13</v>
+        <v>0</v>
       </c>
       <c r="J91" t="n">
-        <v>2.873478648216767e-07</v>
+        <v>0</v>
       </c>
       <c r="K91" t="n">
-        <v>5.047885510272905e-05</v>
+        <v>0</v>
       </c>
       <c r="L91" t="n">
-        <v>7.239883442481702e-11</v>
+        <v>0</v>
       </c>
       <c r="M91" t="n">
-        <v>5.250354986066017e-13</v>
+        <v>0</v>
       </c>
       <c r="N91" t="n">
-        <v>1.231404671601769e-08</v>
+        <v>0</v>
       </c>
       <c r="O91" t="n">
-        <v>2.250215571491093e-05</v>
+        <v>0</v>
       </c>
       <c r="P91" t="n">
-        <v>2.404876306483922e-05</v>
+        <v>0</v>
       </c>
       <c r="Q91" t="n">
-        <v>2.206547667616147e-13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -5530,10 +5530,10 @@
         <v>0</v>
       </c>
       <c r="C93" t="n">
-        <v>9.999999999999974e-07</v>
+        <v>0</v>
       </c>
       <c r="D93" t="n">
-        <v>1.763980120268387e-05</v>
+        <v>0</v>
       </c>
       <c r="E93" t="n">
         <v>0</v>
@@ -5548,7 +5548,7 @@
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>5.324412329054144e-22</v>
+        <v>0</v>
       </c>
       <c r="J93" t="n">
         <v>0</v>
@@ -5560,7 +5560,7 @@
         <v>0</v>
       </c>
       <c r="M93" t="n">
-        <v>7.887435940696315e-12</v>
+        <v>0</v>
       </c>
       <c r="N93" t="n">
         <v>0</v>
@@ -5637,52 +5637,52 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>7.843322698906691</v>
+        <v>7.84332271486945</v>
       </c>
       <c r="C95" t="n">
-        <v>3930.810762</v>
+        <v>3930.81077</v>
       </c>
       <c r="D95" t="n">
-        <v>12958.9119533673</v>
+        <v>12958.91197974132</v>
       </c>
       <c r="E95" t="n">
-        <v>1.151812786366915e-05</v>
+        <v>1.151812788711089e-05</v>
       </c>
       <c r="F95" t="n">
-        <v>3.924235556681295</v>
+        <v>3.924235564667913</v>
       </c>
       <c r="G95" t="n">
-        <v>43.80703978058244</v>
+        <v>43.80703986973867</v>
       </c>
       <c r="H95" t="n">
-        <v>2.724051134522791e-07</v>
+        <v>2.724051140066789e-07</v>
       </c>
       <c r="I95" t="n">
-        <v>8.641179550665565e-05</v>
+        <v>8.641179568252124e-05</v>
       </c>
       <c r="J95" t="n">
-        <v>0.005730667531867807</v>
+        <v>0.005730667543530882</v>
       </c>
       <c r="K95" t="n">
-        <v>0.4391936639316629</v>
+        <v>0.4391936648255114</v>
       </c>
       <c r="L95" t="n">
-        <v>4.091512445542974e-06</v>
+        <v>4.091512453870035e-06</v>
       </c>
       <c r="M95" t="n">
-        <v>0.0005228627541773752</v>
+        <v>0.0005228627552415073</v>
       </c>
       <c r="N95" t="n">
-        <v>10.32322178416444</v>
+        <v>10.3232218051743</v>
       </c>
       <c r="O95" t="n">
-        <v>0.07986051963894228</v>
+        <v>0.07986051980147468</v>
       </c>
       <c r="P95" t="n">
-        <v>1.019646133137129</v>
+        <v>1.019646135212317</v>
       </c>
       <c r="Q95" t="n">
-        <v>1.243831665930911e-05</v>
+        <v>1.243831668462361e-05</v>
       </c>
     </row>
     <row r="96">
@@ -5692,52 +5692,52 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>1.028015896687431e-07</v>
+        <v>1.713359827812385e-08</v>
       </c>
       <c r="C96" t="n">
-        <v>5.99999999999997e-06</v>
+        <v>9.999999999999951e-07</v>
       </c>
       <c r="D96" t="n">
-        <v>0.008492811782259023</v>
+        <v>0.001415468630376504</v>
       </c>
       <c r="E96" t="n">
-        <v>7.122568373597459e-12</v>
+        <v>1.18709472893291e-12</v>
       </c>
       <c r="F96" t="n">
-        <v>1.114126496263571e-09</v>
+        <v>1.856877493772618e-10</v>
       </c>
       <c r="G96" t="n">
-        <v>1.963893675779516e-08</v>
+        <v>3.273156126299194e-09</v>
       </c>
       <c r="H96" t="n">
-        <v>1.351243768280425e-13</v>
+        <v>2.252072947134042e-14</v>
       </c>
       <c r="I96" t="n">
-        <v>5.438604074551482e-11</v>
+        <v>9.06434012425247e-12</v>
       </c>
       <c r="J96" t="n">
-        <v>3.54372444942463e-09</v>
+        <v>5.906207415707717e-10</v>
       </c>
       <c r="K96" t="n">
-        <v>2.715881380750322e-07</v>
+        <v>4.526468967917204e-08</v>
       </c>
       <c r="L96" t="n">
-        <v>2.530105368662008e-12</v>
+        <v>4.216842281103348e-13</v>
       </c>
       <c r="M96" t="n">
-        <v>3.196769611209183e-10</v>
+        <v>5.327949352015305e-11</v>
       </c>
       <c r="N96" t="n">
-        <v>6.633254182851054e-09</v>
+        <v>1.105542363808509e-09</v>
       </c>
       <c r="O96" t="n">
-        <v>4.938406815864184e-08</v>
+        <v>8.230678026440306e-09</v>
       </c>
       <c r="P96" t="n">
-        <v>6.305277546927631e-07</v>
+        <v>1.050879591154605e-07</v>
       </c>
       <c r="Q96" t="n">
-        <v>7.691593799529487e-12</v>
+        <v>1.281932299921581e-12</v>
       </c>
     </row>
     <row r="97">
@@ -5802,52 +5802,52 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>3.437856032878802</v>
+        <v>3.437870134885496</v>
       </c>
       <c r="C98" t="n">
-        <v>1726.240747</v>
+        <v>1726.247828</v>
       </c>
       <c r="D98" t="n">
-        <v>5094.462458226869</v>
+        <v>5094.48335559517</v>
       </c>
       <c r="E98" t="n">
-        <v>4.527741342114073e-06</v>
+        <v>4.52775991480534e-06</v>
       </c>
       <c r="F98" t="n">
-        <v>1.723732406199264</v>
+        <v>1.723739476910108</v>
       </c>
       <c r="G98" t="n">
-        <v>19.24175718654886</v>
+        <v>19.24183611579606</v>
       </c>
       <c r="H98" t="n">
-        <v>1.099717831998395e-07</v>
+        <v>1.09972234301575e-07</v>
       </c>
       <c r="I98" t="n">
-        <v>3.404587507310295e-05</v>
+        <v>3.404601472850259e-05</v>
       </c>
       <c r="J98" t="n">
-        <v>0.002252708131830303</v>
+        <v>0.002252717372387456</v>
       </c>
       <c r="K98" t="n">
-        <v>0.1726457053537589</v>
+        <v>0.1726464135424874</v>
       </c>
       <c r="L98" t="n">
-        <v>1.608361208586016e-06</v>
+        <v>1.60836780604685e-06</v>
       </c>
       <c r="M98" t="n">
-        <v>0.0002070303500479896</v>
+        <v>0.0002070311992817429</v>
       </c>
       <c r="N98" t="n">
-        <v>4.534202243930716</v>
+        <v>4.534220843124452</v>
       </c>
       <c r="O98" t="n">
-        <v>0.03139292953262688</v>
+        <v>0.03139305830570469</v>
       </c>
       <c r="P98" t="n">
-        <v>0.4008198212396873</v>
+        <v>0.4008214653934122</v>
       </c>
       <c r="Q98" t="n">
-        <v>4.889464783795157e-06</v>
+        <v>4.889484840267694e-06</v>
       </c>
     </row>
     <row r="99">
@@ -5857,52 +5857,52 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>3.249200451488972e-09</v>
+        <v>1.624600225744486e-09</v>
       </c>
       <c r="C99" t="n">
-        <v>4e-06</v>
+        <v>2e-06</v>
       </c>
       <c r="D99" t="n">
-        <v>1.248585184188991e-05</v>
+        <v>6.242925920944955e-06</v>
       </c>
       <c r="E99" t="n">
-        <v>1.092645179653643e-14</v>
+        <v>5.463225898268213e-15</v>
       </c>
       <c r="F99" t="n">
-        <v>8.250243869885525e-10</v>
+        <v>4.125121934942762e-10</v>
       </c>
       <c r="G99" t="n">
-        <v>1.573477645704226e-08</v>
+        <v>7.867388228521126e-09</v>
       </c>
       <c r="H99" t="n">
-        <v>2.073283007642123e-16</v>
+        <v>1.036641503821061e-16</v>
       </c>
       <c r="I99" t="n">
-        <v>8.281899513676059e-14</v>
+        <v>4.140949756838029e-14</v>
       </c>
       <c r="J99" t="n">
-        <v>5.436288196316603e-12</v>
+        <v>2.718144098158301e-12</v>
       </c>
       <c r="K99" t="n">
-        <v>4.16632672869534e-10</v>
+        <v>2.08316336434767e-10</v>
       </c>
       <c r="L99" t="n">
-        <v>3.8813350607234e-15</v>
+        <v>1.9406675303617e-15</v>
       </c>
       <c r="M99" t="n">
-        <v>4.899320220850427e-13</v>
+        <v>2.449660110425213e-13</v>
       </c>
       <c r="N99" t="n">
-        <v>2.256263070201403e-09</v>
+        <v>1.128131535100701e-09</v>
       </c>
       <c r="O99" t="n">
-        <v>7.57581551975657e-11</v>
+        <v>3.787907759878285e-11</v>
       </c>
       <c r="P99" t="n">
-        <v>9.672678108036348e-10</v>
+        <v>4.836339054018174e-10</v>
       </c>
       <c r="Q99" t="n">
-        <v>1.179937130552945e-14</v>
+        <v>5.899685652764723e-15</v>
       </c>
     </row>
     <row r="100">
@@ -6627,52 +6627,52 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.02066963826643698</v>
+        <v>0.02077891731812774</v>
       </c>
       <c r="C113" t="n">
-        <v>3.022923</v>
+        <v>3.038905000000001</v>
       </c>
       <c r="D113" t="n">
-        <v>108.6770468030225</v>
+        <v>109.2516153785389</v>
       </c>
       <c r="E113" t="n">
-        <v>0.0004680346280293299</v>
+        <v>0.0004705090970863204</v>
       </c>
       <c r="F113" t="n">
-        <v>0.01180102870669594</v>
+        <v>0.01186341998850841</v>
       </c>
       <c r="G113" t="n">
-        <v>0.06429124464172474</v>
+        <v>0.06463114832827714</v>
       </c>
       <c r="H113" t="n">
-        <v>2.171992802629322e-09</v>
+        <v>2.183475989257503e-09</v>
       </c>
       <c r="I113" t="n">
-        <v>6.80527002351194e-08</v>
+        <v>6.841249049612098e-08</v>
       </c>
       <c r="J113" t="n">
-        <v>0.3355599653224542</v>
+        <v>0.3373340493351081</v>
       </c>
       <c r="K113" t="n">
-        <v>159.6669003542595</v>
+        <v>160.5110490148313</v>
       </c>
       <c r="L113" t="n">
-        <v>4.08657814345814e-05</v>
+        <v>4.108183619974991e-05</v>
       </c>
       <c r="M113" t="n">
-        <v>1.871951718272217e-07</v>
+        <v>1.881848606933101e-07</v>
       </c>
       <c r="N113" t="n">
-        <v>0.03382808334537829</v>
+        <v>0.03400693025217209</v>
       </c>
       <c r="O113" t="n">
-        <v>6.445812022910419</v>
+        <v>6.479890617618309</v>
       </c>
       <c r="P113" t="n">
-        <v>63.97916006586246</v>
+        <v>64.31741378128049</v>
       </c>
       <c r="Q113" t="n">
-        <v>8.158947833854823e-07</v>
+        <v>8.20208366770857e-07</v>
       </c>
     </row>
     <row r="114">
@@ -6682,52 +6682,52 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>0.01461859966905812</v>
+        <v>0.01472138296933441</v>
       </c>
       <c r="C114" t="n">
-        <v>2.137961999999999</v>
+        <v>2.152994</v>
       </c>
       <c r="D114" t="n">
-        <v>76.86183086273924</v>
+        <v>77.40224600647366</v>
       </c>
       <c r="E114" t="n">
-        <v>0.0003310174455025316</v>
+        <v>0.0003333448274863059</v>
       </c>
       <c r="F114" t="n">
-        <v>0.008346276413863369</v>
+        <v>0.008404959041081813</v>
       </c>
       <c r="G114" t="n">
-        <v>0.04546997656794802</v>
+        <v>0.04578967574303599</v>
       </c>
       <c r="H114" t="n">
-        <v>1.536141700035019e-09</v>
+        <v>1.546942304552278e-09</v>
       </c>
       <c r="I114" t="n">
-        <v>4.813026567334906e-08</v>
+        <v>4.846866932767117e-08</v>
       </c>
       <c r="J114" t="n">
-        <v>0.2373247530885588</v>
+        <v>0.238993382226227</v>
       </c>
       <c r="K114" t="n">
-        <v>112.924399865691</v>
+        <v>113.7183707495426</v>
       </c>
       <c r="L114" t="n">
-        <v>2.890231997554767e-05</v>
+        <v>2.910553204099713e-05</v>
       </c>
       <c r="M114" t="n">
-        <v>1.323937672081197e-07</v>
+        <v>1.333246271152053e-07</v>
       </c>
       <c r="N114" t="n">
-        <v>0.0239249086811843</v>
+        <v>0.0240931245930179</v>
       </c>
       <c r="O114" t="n">
-        <v>4.558799931101636</v>
+        <v>4.590852830341342</v>
       </c>
       <c r="P114" t="n">
-        <v>45.24925478178949</v>
+        <v>45.56740206311623</v>
       </c>
       <c r="Q114" t="n">
-        <v>5.770415068052981e-07</v>
+        <v>5.810986827187603e-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>